<commit_message>
Atulizando os preços 16/09
</commit_message>
<xml_diff>
--- a/data/ProdutosFomatodos.xlsx
+++ b/data/ProdutosFomatodos.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="6"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="16"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="promoçoes"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3766" uniqueCount="1141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3758" uniqueCount="1141">
   <si>
     <t>produto_grupo</t>
   </si>
@@ -4701,7 +4701,7 @@
         <v>15</v>
       </c>
       <c r="G2" s="4">
-        <v>300</v>
+        <v>310</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
@@ -5046,7 +5046,7 @@
         <v>15</v>
       </c>
       <c r="G17" s="4">
-        <v>675</v>
+        <v>850</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
@@ -5069,7 +5069,7 @@
         <v>10</v>
       </c>
       <c r="G18" s="5">
-        <v>337.5</v>
+        <v>425</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
@@ -5459,7 +5459,7 @@
         <v>10</v>
       </c>
       <c r="G9" s="4">
-        <v>103.5</v>
+        <v>108.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
@@ -5482,7 +5482,7 @@
         <v>158</v>
       </c>
       <c r="G10" s="4">
-        <v>500</v>
+        <v>525</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
@@ -5689,7 +5689,7 @@
         <v>10</v>
       </c>
       <c r="G19" s="5">
-        <v>162.5</v>
+        <v>202.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
@@ -5712,7 +5712,7 @@
         <v>15</v>
       </c>
       <c r="G20" s="4">
-        <v>325</v>
+        <v>405</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
@@ -5965,7 +5965,7 @@
         <v>158</v>
       </c>
       <c r="G31" s="4">
-        <v>1725</v>
+        <v>1850</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="19.5">
@@ -5988,7 +5988,7 @@
         <v>158</v>
       </c>
       <c r="G32" s="4">
-        <v>348.5</v>
+        <v>373.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="19.5">
@@ -6070,7 +6070,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:G119"/>
+  <dimension ref="A1:G120"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="6" width="30.005" customWidth="1" bestFit="1"/>
@@ -6516,7 +6516,7 @@
         <v>158</v>
       </c>
       <c r="G19" s="4">
-        <v>450</v>
+        <v>575</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
@@ -6539,7 +6539,7 @@
         <v>10</v>
       </c>
       <c r="G20" s="4">
-        <v>56</v>
+        <v>71</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
@@ -6608,7 +6608,7 @@
         <v>158</v>
       </c>
       <c r="G23" s="4">
-        <v>190</v>
+        <v>180</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="19.5">
@@ -6631,7 +6631,7 @@
         <v>10</v>
       </c>
       <c r="G24" s="4">
-        <v>200</v>
+        <v>260</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="19.5">
@@ -6746,7 +6746,7 @@
         <v>158</v>
       </c>
       <c r="G29" s="4">
-        <v>627.5</v>
+        <v>595</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="19.5">
@@ -8103,7 +8103,7 @@
         <v>10</v>
       </c>
       <c r="G88" s="5">
-        <v>115</v>
+        <v>127</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18.75">
@@ -8126,30 +8126,30 @@
         <v>158</v>
       </c>
       <c r="G89" s="4">
-        <v>280</v>
+        <v>310</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18.75">
       <c r="A90" s="3" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="C90" s="4">
-        <v>4378</v>
+        <v>4225</v>
       </c>
       <c r="D90" s="4">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E90" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F90" s="3" t="s">
-        <v>158</v>
+        <v>10</v>
       </c>
       <c r="G90" s="4">
-        <v>430</v>
+        <v>775</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18.75">
@@ -8160,10 +8160,10 @@
         <v>448</v>
       </c>
       <c r="C91" s="4">
-        <v>4379</v>
+        <v>4378</v>
       </c>
       <c r="D91" s="4">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E91" s="3" t="s">
         <v>29</v>
@@ -8172,30 +8172,30 @@
         <v>158</v>
       </c>
       <c r="G91" s="4">
-        <v>43</v>
+        <v>430</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18.75">
       <c r="A92" s="3" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="C92" s="4">
-        <v>3524</v>
+        <v>4379</v>
       </c>
       <c r="D92" s="4">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="E92" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F92" s="3" t="s">
-        <v>9</v>
+        <v>158</v>
       </c>
       <c r="G92" s="4">
-        <v>350</v>
+        <v>43</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18.75">
@@ -8206,10 +8206,10 @@
         <v>450</v>
       </c>
       <c r="C93" s="4">
-        <v>3523</v>
+        <v>3524</v>
       </c>
       <c r="D93" s="4">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="E93" s="3" t="s">
         <v>29</v>
@@ -8218,30 +8218,30 @@
         <v>9</v>
       </c>
       <c r="G93" s="4">
-        <v>72</v>
+        <v>350</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18.75">
       <c r="A94" s="3" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="C94" s="4">
-        <v>3521</v>
+        <v>3523</v>
       </c>
       <c r="D94" s="4">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="E94" s="3" t="s">
-        <v>453</v>
+        <v>29</v>
       </c>
       <c r="F94" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="G94" s="4">
-        <v>158</v>
+        <v>72</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18.75">
@@ -8252,53 +8252,53 @@
         <v>452</v>
       </c>
       <c r="C95" s="4">
-        <v>3522</v>
+        <v>3521</v>
       </c>
       <c r="D95" s="4">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E95" s="3" t="s">
-        <v>74</v>
+        <v>453</v>
       </c>
       <c r="F95" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="G95" s="5">
-        <v>216.5</v>
+      <c r="G95" s="4">
+        <v>158</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18.75">
       <c r="A96" s="3" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="C96" s="4">
-        <v>64</v>
+        <v>3522</v>
       </c>
       <c r="D96" s="4">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E96" s="3" t="s">
-        <v>38</v>
+        <v>74</v>
       </c>
       <c r="F96" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="G96" s="4">
-        <v>132</v>
+      <c r="G96" s="5">
+        <v>216.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18.75">
       <c r="A97" s="3" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="C97" s="4">
-        <v>90</v>
+        <v>64</v>
       </c>
       <c r="D97" s="4">
         <v>8</v>
@@ -8315,25 +8315,25 @@
     </row>
     <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="18.75">
       <c r="A98" s="3" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="C98" s="4">
-        <v>3637</v>
+        <v>90</v>
       </c>
       <c r="D98" s="4">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="E98" s="3" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="F98" s="3" t="s">
-        <v>158</v>
+        <v>15</v>
       </c>
       <c r="G98" s="4">
-        <v>375</v>
+        <v>132</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="18.75">
@@ -8344,10 +8344,10 @@
         <v>459</v>
       </c>
       <c r="C99" s="4">
-        <v>2805</v>
+        <v>3637</v>
       </c>
       <c r="D99" s="4">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E99" s="3" t="s">
         <v>29</v>
@@ -8356,7 +8356,7 @@
         <v>158</v>
       </c>
       <c r="G99" s="4">
-        <v>150</v>
+        <v>375</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="18.75">
@@ -8367,42 +8367,42 @@
         <v>459</v>
       </c>
       <c r="C100" s="4">
-        <v>2427</v>
+        <v>2805</v>
       </c>
       <c r="D100" s="4">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E100" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F100" s="3" t="s">
-        <v>10</v>
+        <v>158</v>
       </c>
       <c r="G100" s="4">
-        <v>46</v>
+        <v>150</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="18.75">
       <c r="A101" s="3" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="C101" s="4">
-        <v>3437</v>
+        <v>2427</v>
       </c>
       <c r="D101" s="4">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E101" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F101" s="3" t="s">
-        <v>158</v>
+        <v>10</v>
       </c>
       <c r="G101" s="4">
-        <v>350</v>
+        <v>46</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="18.75">
@@ -8413,53 +8413,53 @@
         <v>461</v>
       </c>
       <c r="C102" s="4">
-        <v>3396</v>
+        <v>3437</v>
       </c>
       <c r="D102" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E102" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F102" s="3" t="s">
-        <v>10</v>
+        <v>158</v>
       </c>
       <c r="G102" s="4">
-        <v>178.5</v>
+        <v>350</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="18.75">
       <c r="A103" s="3" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="C103" s="4">
-        <v>3395</v>
+        <v>3396</v>
       </c>
       <c r="D103" s="4">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E103" s="3" t="s">
-        <v>464</v>
+        <v>29</v>
       </c>
       <c r="F103" s="3" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G103" s="4">
-        <v>54</v>
+        <v>178.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="104" customHeight="1" ht="18.75">
       <c r="A104" s="3" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="C104" s="4">
-        <v>3490</v>
+        <v>3395</v>
       </c>
       <c r="D104" s="4">
         <v>12</v>
@@ -8471,41 +8471,41 @@
         <v>15</v>
       </c>
       <c r="G104" s="4">
-        <v>169</v>
+        <v>54</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="105" customHeight="1" ht="18.75">
       <c r="A105" s="3" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="C105" s="4">
-        <v>458</v>
+        <v>3490</v>
       </c>
       <c r="D105" s="4">
         <v>12</v>
       </c>
       <c r="E105" s="3" t="s">
-        <v>314</v>
+        <v>464</v>
       </c>
       <c r="F105" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="G105" s="5">
-        <v>269.5</v>
+      <c r="G105" s="4">
+        <v>169</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="106" customHeight="1" ht="18.75">
       <c r="A106" s="3" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="C106" s="4">
-        <v>2641</v>
+        <v>458</v>
       </c>
       <c r="D106" s="4">
         <v>12</v>
@@ -8516,19 +8516,19 @@
       <c r="F106" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="G106" s="4">
-        <v>222</v>
+      <c r="G106" s="5">
+        <v>269.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="107" customHeight="1" ht="18.75">
       <c r="A107" s="3" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="C107" s="4">
-        <v>4293</v>
+        <v>2641</v>
       </c>
       <c r="D107" s="4">
         <v>12</v>
@@ -8540,30 +8540,30 @@
         <v>15</v>
       </c>
       <c r="G107" s="4">
-        <v>210</v>
+        <v>222</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="108" customHeight="1" ht="18.75">
       <c r="A108" s="3" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="C108" s="4">
-        <v>2396</v>
+        <v>4293</v>
       </c>
       <c r="D108" s="4">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="E108" s="3" t="s">
-        <v>29</v>
+        <v>314</v>
       </c>
       <c r="F108" s="3" t="s">
-        <v>158</v>
+        <v>15</v>
       </c>
       <c r="G108" s="4">
-        <v>575</v>
+        <v>210</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="109" customHeight="1" ht="18.75">
@@ -8574,33 +8574,33 @@
         <v>474</v>
       </c>
       <c r="C109" s="4">
-        <v>2426</v>
+        <v>2396</v>
       </c>
       <c r="D109" s="4">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E109" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F109" s="3" t="s">
-        <v>10</v>
+        <v>158</v>
       </c>
       <c r="G109" s="4">
-        <v>118.5</v>
+        <v>675</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="110" customHeight="1" ht="18.75">
       <c r="A110" s="3" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="C110" s="4">
-        <v>4335</v>
+        <v>2426</v>
       </c>
       <c r="D110" s="4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E110" s="3" t="s">
         <v>29</v>
@@ -8609,18 +8609,18 @@
         <v>10</v>
       </c>
       <c r="G110" s="4">
-        <v>510</v>
+        <v>137</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="111" customHeight="1" ht="18.75">
       <c r="A111" s="3" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="C111" s="4">
-        <v>4477</v>
+        <v>4335</v>
       </c>
       <c r="D111" s="4">
         <v>3</v>
@@ -8632,18 +8632,18 @@
         <v>10</v>
       </c>
       <c r="G111" s="4">
-        <v>252</v>
+        <v>510</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="112" customHeight="1" ht="18.75">
       <c r="A112" s="3" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="C112" s="4">
-        <v>4479</v>
+        <v>4477</v>
       </c>
       <c r="D112" s="4">
         <v>3</v>
@@ -8660,13 +8660,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="113" customHeight="1" ht="18.75">
       <c r="A113" s="3" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="C113" s="4">
-        <v>4478</v>
+        <v>4479</v>
       </c>
       <c r="D113" s="4">
         <v>3</v>
@@ -8683,25 +8683,25 @@
     </row>
     <row x14ac:dyDescent="0.25" r="114" customHeight="1" ht="18.75">
       <c r="A114" s="3" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="C114" s="4">
-        <v>2646</v>
+        <v>4478</v>
       </c>
       <c r="D114" s="4">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E114" s="3" t="s">
-        <v>485</v>
+        <v>29</v>
       </c>
       <c r="F114" s="3" t="s">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="G114" s="4">
-        <v>53</v>
+        <v>252</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="115" customHeight="1" ht="18.75">
@@ -8712,19 +8712,19 @@
         <v>484</v>
       </c>
       <c r="C115" s="4">
-        <v>2645</v>
+        <v>2646</v>
       </c>
       <c r="D115" s="4">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E115" s="3" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="F115" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="G115" s="5">
-        <v>81.5</v>
+      <c r="G115" s="4">
+        <v>53</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="116" customHeight="1" ht="18.75">
@@ -8735,87 +8735,110 @@
         <v>484</v>
       </c>
       <c r="C116" s="4">
-        <v>2638</v>
+        <v>2645</v>
       </c>
       <c r="D116" s="4">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E116" s="3" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="F116" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="G116" s="4">
-        <v>70</v>
+      <c r="G116" s="5">
+        <v>81.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="117" customHeight="1" ht="18.75">
       <c r="A117" s="3" t="s">
-        <v>488</v>
+        <v>483</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>489</v>
+        <v>484</v>
       </c>
       <c r="C117" s="4">
-        <v>4294</v>
+        <v>2638</v>
       </c>
       <c r="D117" s="4">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="E117" s="3" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="F117" s="3" t="s">
         <v>49</v>
       </c>
       <c r="G117" s="4">
-        <v>150</v>
+        <v>70</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="118" customHeight="1" ht="18.75">
       <c r="A118" s="3" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="C118" s="4">
-        <v>4314</v>
+        <v>4294</v>
       </c>
       <c r="D118" s="4">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E118" s="3" t="s">
-        <v>74</v>
+        <v>490</v>
       </c>
       <c r="F118" s="3" t="s">
-        <v>15</v>
+        <v>49</v>
       </c>
       <c r="G118" s="4">
-        <v>252</v>
+        <v>150</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="119" customHeight="1" ht="18.75">
       <c r="A119" s="3" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="C119" s="4">
-        <v>4315</v>
+        <v>4314</v>
       </c>
       <c r="D119" s="4">
         <v>15</v>
       </c>
       <c r="E119" s="3" t="s">
-        <v>495</v>
+        <v>74</v>
       </c>
       <c r="F119" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G119" s="4">
+        <v>252</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="120" customHeight="1" ht="18.75">
+      <c r="A120" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="B120" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="C120" s="4">
+        <v>4315</v>
+      </c>
+      <c r="D120" s="4">
+        <v>15</v>
+      </c>
+      <c r="E120" s="3" t="s">
+        <v>495</v>
+      </c>
+      <c r="F120" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G120" s="4">
         <v>450</v>
       </c>
     </row>
@@ -10113,7 +10136,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:G130"/>
+  <dimension ref="A1:G128"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="6" width="30.005" customWidth="1" bestFit="1"/>
@@ -12272,30 +12295,30 @@
         <v>187</v>
       </c>
       <c r="C94" s="4">
-        <v>4629</v>
+        <v>4643</v>
       </c>
       <c r="D94" s="4">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E94" s="3" t="s">
         <v>165</v>
       </c>
       <c r="F94" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G94" s="4">
-        <v>195</v>
+        <v>188</v>
+      </c>
+      <c r="G94" s="5">
+        <v>97.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18.75">
       <c r="A95" s="3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="C95" s="4">
-        <v>4643</v>
+        <v>4687</v>
       </c>
       <c r="D95" s="4">
         <v>6</v>
@@ -12304,90 +12327,90 @@
         <v>165</v>
       </c>
       <c r="F95" s="3" t="s">
-        <v>188</v>
+        <v>149</v>
       </c>
       <c r="G95" s="5">
-        <v>97.5</v>
+        <v>64</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18.75">
       <c r="A96" s="3" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C96" s="4">
-        <v>4630</v>
+        <v>4644</v>
       </c>
       <c r="D96" s="4">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E96" s="3" t="s">
         <v>165</v>
       </c>
       <c r="F96" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G96" s="5">
-        <v>127.5</v>
+        <v>149</v>
+      </c>
+      <c r="G96" s="4">
+        <v>57</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18.75">
       <c r="A97" s="3" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="C97" s="4">
-        <v>4687</v>
+        <v>4104</v>
       </c>
       <c r="D97" s="4">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E97" s="3" t="s">
         <v>165</v>
       </c>
       <c r="F97" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="G97" s="5">
-        <v>64</v>
+        <v>49</v>
+      </c>
+      <c r="G97" s="4">
+        <v>77</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="18.75">
       <c r="A98" s="3" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="C98" s="4">
-        <v>4644</v>
+        <v>4101</v>
       </c>
       <c r="D98" s="4">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E98" s="3" t="s">
         <v>165</v>
       </c>
       <c r="F98" s="3" t="s">
-        <v>149</v>
+        <v>49</v>
       </c>
       <c r="G98" s="4">
-        <v>113</v>
+        <v>77</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="18.75">
       <c r="A99" s="3" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C99" s="4">
-        <v>4104</v>
+        <v>4105</v>
       </c>
       <c r="D99" s="4">
         <v>10</v>
@@ -12404,36 +12427,36 @@
     </row>
     <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="18.75">
       <c r="A100" s="3" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="C100" s="4">
-        <v>4101</v>
+        <v>3705</v>
       </c>
       <c r="D100" s="4">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E100" s="3" t="s">
-        <v>165</v>
+        <v>201</v>
       </c>
       <c r="F100" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="G100" s="4">
-        <v>77</v>
+      <c r="G100" s="5">
+        <v>123.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="18.75">
       <c r="A101" s="3" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="C101" s="4">
-        <v>4105</v>
+        <v>3823</v>
       </c>
       <c r="D101" s="4">
         <v>10</v>
@@ -12442,7 +12465,7 @@
         <v>165</v>
       </c>
       <c r="F101" s="3" t="s">
-        <v>49</v>
+        <v>15</v>
       </c>
       <c r="G101" s="4">
         <v>77</v>
@@ -12450,197 +12473,197 @@
     </row>
     <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="18.75">
       <c r="A102" s="3" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="C102" s="4">
-        <v>3705</v>
+        <v>4641</v>
       </c>
       <c r="D102" s="4">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E102" s="3" t="s">
-        <v>201</v>
+        <v>165</v>
       </c>
       <c r="F102" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="G102" s="5">
-        <v>123.5</v>
+        <v>10</v>
+      </c>
+      <c r="G102" s="4">
+        <v>72</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="18.75">
       <c r="A103" s="3" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="C103" s="4">
-        <v>3823</v>
+        <v>4583</v>
       </c>
       <c r="D103" s="4">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E103" s="3" t="s">
         <v>165</v>
       </c>
       <c r="F103" s="3" t="s">
-        <v>15</v>
+        <v>49</v>
       </c>
       <c r="G103" s="4">
-        <v>77</v>
+        <v>144</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="104" customHeight="1" ht="18.75">
       <c r="A104" s="3" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="C104" s="4">
-        <v>4641</v>
+        <v>4308</v>
       </c>
       <c r="D104" s="4">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E104" s="3" t="s">
-        <v>165</v>
+        <v>209</v>
       </c>
       <c r="F104" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G104" s="4">
-        <v>72</v>
+      <c r="G104" s="5">
+        <v>68.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="105" customHeight="1" ht="18.75">
       <c r="A105" s="3" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="C105" s="4">
-        <v>4583</v>
+        <v>4309</v>
       </c>
       <c r="D105" s="4">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E105" s="3" t="s">
-        <v>165</v>
+        <v>209</v>
       </c>
       <c r="F105" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="G105" s="4">
-        <v>144</v>
+        <v>149</v>
+      </c>
+      <c r="G105" s="5">
+        <v>68.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="106" customHeight="1" ht="18.75">
       <c r="A106" s="3" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="C106" s="4">
-        <v>4308</v>
+        <v>4635</v>
       </c>
       <c r="D106" s="4">
         <v>10</v>
       </c>
       <c r="E106" s="3" t="s">
-        <v>209</v>
+        <v>74</v>
       </c>
       <c r="F106" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G106" s="5">
-        <v>68.5</v>
+        <v>149</v>
+      </c>
+      <c r="G106" s="4">
+        <v>177</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="107" customHeight="1" ht="18.75">
       <c r="A107" s="3" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="C107" s="4">
-        <v>4309</v>
-      </c>
-      <c r="D107" s="4">
-        <v>10</v>
+        <v>4412</v>
+      </c>
+      <c r="D107" s="5">
+        <v>2.5</v>
       </c>
       <c r="E107" s="3" t="s">
-        <v>209</v>
+        <v>29</v>
       </c>
       <c r="F107" s="3" t="s">
         <v>149</v>
       </c>
       <c r="G107" s="5">
-        <v>68.5</v>
+        <v>75.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="108" customHeight="1" ht="18.75">
       <c r="A108" s="3" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="C108" s="4">
-        <v>4635</v>
+        <v>4413</v>
       </c>
       <c r="D108" s="4">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E108" s="3" t="s">
-        <v>74</v>
+        <v>29</v>
       </c>
       <c r="F108" s="3" t="s">
-        <v>149</v>
+        <v>10</v>
       </c>
       <c r="G108" s="4">
-        <v>177</v>
+        <v>496</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="109" customHeight="1" ht="18.75">
       <c r="A109" s="3" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C109" s="4">
-        <v>4412</v>
-      </c>
-      <c r="D109" s="5">
-        <v>2.5</v>
+        <v>4414</v>
+      </c>
+      <c r="D109" s="4">
+        <v>5</v>
       </c>
       <c r="E109" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F109" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="G109" s="5">
-        <v>75.5</v>
+        <v>10</v>
+      </c>
+      <c r="G109" s="4">
+        <v>101</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="110" customHeight="1" ht="18.75">
       <c r="A110" s="3" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C110" s="4">
-        <v>4413</v>
+        <v>4415</v>
       </c>
       <c r="D110" s="4">
         <v>25</v>
@@ -12652,18 +12675,18 @@
         <v>10</v>
       </c>
       <c r="G110" s="4">
-        <v>496</v>
+        <v>424</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="111" customHeight="1" ht="18.75">
       <c r="A111" s="3" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C111" s="4">
-        <v>4414</v>
+        <v>4416</v>
       </c>
       <c r="D111" s="4">
         <v>5</v>
@@ -12675,87 +12698,87 @@
         <v>10</v>
       </c>
       <c r="G111" s="4">
-        <v>101</v>
+        <v>88</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="112" customHeight="1" ht="18.75">
       <c r="A112" s="3" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C112" s="4">
-        <v>4415</v>
+        <v>4475</v>
       </c>
       <c r="D112" s="4">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E112" s="3" t="s">
-        <v>29</v>
+        <v>222</v>
       </c>
       <c r="F112" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G112" s="4">
-        <v>424</v>
+        <v>9</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="113" customHeight="1" ht="18.75">
       <c r="A113" s="3" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="C113" s="4">
-        <v>4416</v>
+        <v>4354</v>
       </c>
       <c r="D113" s="4">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E113" s="3" t="s">
-        <v>29</v>
+        <v>222</v>
       </c>
       <c r="F113" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G113" s="4">
-        <v>88</v>
+        <v>9</v>
+      </c>
+      <c r="G113" s="5">
+        <v>79.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="114" customHeight="1" ht="18.75">
       <c r="A114" s="3" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="C114" s="4">
-        <v>4475</v>
+        <v>4445</v>
       </c>
       <c r="D114" s="4">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E114" s="3" t="s">
         <v>222</v>
       </c>
       <c r="F114" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G114" s="4">
-        <v>9</v>
+        <v>15</v>
+      </c>
+      <c r="G114" s="5">
+        <v>79.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="115" customHeight="1" ht="18.75">
       <c r="A115" s="3" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="C115" s="4">
-        <v>4354</v>
+        <v>4353</v>
       </c>
       <c r="D115" s="4">
         <v>12</v>
@@ -12764,7 +12787,7 @@
         <v>222</v>
       </c>
       <c r="F115" s="3" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="G115" s="5">
         <v>79.5</v>
@@ -12772,13 +12795,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="116" customHeight="1" ht="18.75">
       <c r="A116" s="3" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="C116" s="4">
-        <v>4445</v>
+        <v>4350</v>
       </c>
       <c r="D116" s="4">
         <v>12</v>
@@ -12795,13 +12818,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="117" customHeight="1" ht="18.75">
       <c r="A117" s="3" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="C117" s="4">
-        <v>4353</v>
+        <v>4352</v>
       </c>
       <c r="D117" s="4">
         <v>12</v>
@@ -12818,13 +12841,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="118" customHeight="1" ht="18.75">
       <c r="A118" s="3" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="C118" s="4">
-        <v>4350</v>
+        <v>4349</v>
       </c>
       <c r="D118" s="4">
         <v>12</v>
@@ -12841,13 +12864,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="119" customHeight="1" ht="18.75">
       <c r="A119" s="3" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="C119" s="4">
-        <v>4352</v>
+        <v>4351</v>
       </c>
       <c r="D119" s="4">
         <v>12</v>
@@ -12864,13 +12887,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="120" customHeight="1" ht="18.75">
       <c r="A120" s="3" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="C120" s="4">
-        <v>4349</v>
+        <v>4581</v>
       </c>
       <c r="D120" s="4">
         <v>12</v>
@@ -12887,231 +12910,185 @@
     </row>
     <row x14ac:dyDescent="0.25" r="121" customHeight="1" ht="18.75">
       <c r="A121" s="3" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="C121" s="4">
-        <v>4351</v>
+        <v>4096</v>
       </c>
       <c r="D121" s="4">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E121" s="3" t="s">
-        <v>222</v>
+        <v>29</v>
       </c>
       <c r="F121" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G121" s="5">
-        <v>79.5</v>
+        <v>10</v>
+      </c>
+      <c r="G121" s="4">
+        <v>79</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="122" customHeight="1" ht="18.75">
       <c r="A122" s="3" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C122" s="4">
-        <v>4581</v>
+        <v>4582</v>
       </c>
       <c r="D122" s="4">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="E122" s="3" t="s">
-        <v>222</v>
+        <v>243</v>
       </c>
       <c r="F122" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G122" s="5">
-        <v>79.5</v>
+        <v>10</v>
+      </c>
+      <c r="G122" s="4">
+        <v>45</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="123" customHeight="1" ht="18.75">
       <c r="A123" s="3" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="C123" s="4">
-        <v>4096</v>
+        <v>4123</v>
       </c>
       <c r="D123" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E123" s="3" t="s">
-        <v>29</v>
+        <v>201</v>
       </c>
       <c r="F123" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G123" s="4">
-        <v>79</v>
+        <v>60</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="124" customHeight="1" ht="18.75">
       <c r="A124" s="3" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="B124" s="3" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="C124" s="4">
-        <v>4582</v>
+        <v>4306</v>
       </c>
       <c r="D124" s="4">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E124" s="3" t="s">
-        <v>243</v>
+        <v>165</v>
       </c>
       <c r="F124" s="3" t="s">
-        <v>10</v>
+        <v>149</v>
       </c>
       <c r="G124" s="4">
-        <v>45</v>
+        <v>81</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="125" customHeight="1" ht="18.75">
       <c r="A125" s="3" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="B125" s="3" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="C125" s="4">
-        <v>4123</v>
+        <v>4307</v>
       </c>
       <c r="D125" s="4">
         <v>10</v>
       </c>
       <c r="E125" s="3" t="s">
-        <v>201</v>
+        <v>165</v>
       </c>
       <c r="F125" s="3" t="s">
-        <v>10</v>
+        <v>149</v>
       </c>
       <c r="G125" s="4">
-        <v>60</v>
+        <v>81</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="126" customHeight="1" ht="18.75">
       <c r="A126" s="3" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="C126" s="4">
-        <v>4306</v>
+        <v>2659</v>
       </c>
       <c r="D126" s="4">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E126" s="3" t="s">
-        <v>165</v>
+        <v>252</v>
       </c>
       <c r="F126" s="3" t="s">
-        <v>149</v>
+        <v>49</v>
       </c>
       <c r="G126" s="4">
-        <v>81</v>
+        <v>30</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="127" customHeight="1" ht="18.75">
       <c r="A127" s="3" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C127" s="4">
-        <v>4307</v>
+        <v>2621</v>
       </c>
       <c r="D127" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E127" s="3" t="s">
-        <v>165</v>
+        <v>253</v>
       </c>
       <c r="F127" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="G127" s="4">
-        <v>81</v>
+        <v>49</v>
+      </c>
+      <c r="G127" s="5">
+        <v>25.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="128" customHeight="1" ht="18.75">
       <c r="A128" s="3" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="B128" s="3" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="C128" s="4">
-        <v>2659</v>
+        <v>3656</v>
       </c>
       <c r="D128" s="4">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E128" s="3" t="s">
-        <v>252</v>
+        <v>165</v>
       </c>
       <c r="F128" s="3" t="s">
         <v>49</v>
       </c>
       <c r="G128" s="4">
-        <v>30</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="129" customHeight="1" ht="18.75">
-      <c r="A129" s="3" t="s">
-        <v>250</v>
-      </c>
-      <c r="B129" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="C129" s="4">
-        <v>2621</v>
-      </c>
-      <c r="D129" s="4">
-        <v>5</v>
-      </c>
-      <c r="E129" s="3" t="s">
-        <v>253</v>
-      </c>
-      <c r="F129" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="G129" s="5">
-        <v>25.5</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="130" customHeight="1" ht="18.75">
-      <c r="A130" s="3" t="s">
-        <v>254</v>
-      </c>
-      <c r="B130" s="3" t="s">
-        <v>255</v>
-      </c>
-      <c r="C130" s="4">
-        <v>3656</v>
-      </c>
-      <c r="D130" s="4">
-        <v>5</v>
-      </c>
-      <c r="E130" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="F130" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="G130" s="4">
         <v>27</v>
       </c>
     </row>
@@ -14421,7 +14398,7 @@
         <v>158</v>
       </c>
       <c r="G40" s="4">
-        <v>195</v>
+        <v>215</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
@@ -14444,7 +14421,7 @@
         <v>10</v>
       </c>
       <c r="G41" s="4">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
@@ -14467,7 +14444,7 @@
         <v>10</v>
       </c>
       <c r="G42" s="4">
-        <v>80</v>
+        <v>76</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
@@ -14490,7 +14467,7 @@
         <v>158</v>
       </c>
       <c r="G43" s="4">
-        <v>200</v>
+        <v>190</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
@@ -14513,7 +14490,7 @@
         <v>10</v>
       </c>
       <c r="G44" s="4">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
@@ -14536,7 +14513,7 @@
         <v>10</v>
       </c>
       <c r="G45" s="4">
-        <v>80</v>
+        <v>76</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
@@ -14559,7 +14536,7 @@
         <v>158</v>
       </c>
       <c r="G46" s="4">
-        <v>200</v>
+        <v>190</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
@@ -14582,7 +14559,7 @@
         <v>10</v>
       </c>
       <c r="G47" s="4">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
@@ -14812,7 +14789,7 @@
         <v>15</v>
       </c>
       <c r="G57" s="5">
-        <v>833.5</v>
+        <v>850.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="19.5">
@@ -14835,7 +14812,7 @@
         <v>15</v>
       </c>
       <c r="G58" s="4">
-        <v>1667</v>
+        <v>1701</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="19.5">
@@ -14858,7 +14835,7 @@
         <v>10</v>
       </c>
       <c r="G59" s="4">
-        <v>371</v>
+        <v>378.6</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="19.5">
@@ -14881,7 +14858,7 @@
         <v>15</v>
       </c>
       <c r="G60" s="5">
-        <v>833.5</v>
+        <v>850.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="19.5">
@@ -14904,7 +14881,7 @@
         <v>15</v>
       </c>
       <c r="G61" s="4">
-        <v>1667</v>
+        <v>1701</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="19.5">
@@ -14927,7 +14904,7 @@
         <v>10</v>
       </c>
       <c r="G62" s="4">
-        <v>371</v>
+        <v>378.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="19.5">
@@ -18111,7 +18088,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:G72"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="6" width="30.005" customWidth="1" bestFit="1"/>
@@ -18695,7 +18672,7 @@
         <v>10</v>
       </c>
       <c r="G25" s="4">
-        <v>270</v>
+        <v>330</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
@@ -18718,7 +18695,7 @@
         <v>10</v>
       </c>
       <c r="G26" s="4">
-        <v>138.5</v>
+        <v>165</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
@@ -18787,7 +18764,7 @@
         <v>158</v>
       </c>
       <c r="G29" s="4">
-        <v>675</v>
+        <v>925</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
@@ -18798,10 +18775,10 @@
         <v>893</v>
       </c>
       <c r="C30" s="4">
-        <v>4676</v>
+        <v>4163</v>
       </c>
       <c r="D30" s="4">
-        <v>12.5</v>
+        <v>10</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>29</v>
@@ -18810,7 +18787,7 @@
         <v>158</v>
       </c>
       <c r="G30" s="4">
-        <v>337.5</v>
+        <v>370</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
@@ -18821,33 +18798,33 @@
         <v>893</v>
       </c>
       <c r="C31" s="4">
-        <v>4163</v>
+        <v>4117</v>
       </c>
       <c r="D31" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>158</v>
+        <v>10</v>
       </c>
       <c r="G31" s="4">
-        <v>270</v>
+        <v>187</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
       <c r="A32" s="3" t="s">
-        <v>892</v>
+        <v>894</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>893</v>
+        <v>895</v>
       </c>
       <c r="C32" s="4">
-        <v>4117</v>
+        <v>3738</v>
       </c>
       <c r="D32" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>29</v>
@@ -18856,7 +18833,7 @@
         <v>10</v>
       </c>
       <c r="G32" s="4">
-        <v>138.5</v>
+        <v>100</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
@@ -18867,10 +18844,10 @@
         <v>895</v>
       </c>
       <c r="C33" s="4">
-        <v>3738</v>
+        <v>4317</v>
       </c>
       <c r="D33" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E33" s="3" t="s">
         <v>29</v>
@@ -18879,21 +18856,21 @@
         <v>10</v>
       </c>
       <c r="G33" s="4">
-        <v>100</v>
+        <v>52</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
       <c r="A34" s="3" t="s">
-        <v>894</v>
+        <v>896</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>895</v>
+        <v>897</v>
       </c>
       <c r="C34" s="4">
-        <v>4317</v>
+        <v>2924</v>
       </c>
       <c r="D34" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>29</v>
@@ -18902,7 +18879,7 @@
         <v>10</v>
       </c>
       <c r="G34" s="4">
-        <v>52</v>
+        <v>168</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
@@ -18913,10 +18890,10 @@
         <v>897</v>
       </c>
       <c r="C35" s="4">
-        <v>2924</v>
+        <v>3078</v>
       </c>
       <c r="D35" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>29</v>
@@ -18925,30 +18902,30 @@
         <v>10</v>
       </c>
       <c r="G35" s="4">
-        <v>168</v>
+        <v>86</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
       <c r="A36" s="3" t="s">
-        <v>896</v>
+        <v>898</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>897</v>
+        <v>899</v>
       </c>
       <c r="C36" s="4">
-        <v>3078</v>
+        <v>2348</v>
       </c>
       <c r="D36" s="4">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>10</v>
+        <v>158</v>
       </c>
       <c r="G36" s="4">
-        <v>86</v>
+        <v>140</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
@@ -18959,10 +18936,10 @@
         <v>899</v>
       </c>
       <c r="C37" s="4">
-        <v>2348</v>
+        <v>2538</v>
       </c>
       <c r="D37" s="4">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>29</v>
@@ -18971,18 +18948,18 @@
         <v>158</v>
       </c>
       <c r="G37" s="4">
-        <v>160</v>
+        <v>30</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
       <c r="A38" s="3" t="s">
-        <v>898</v>
+        <v>900</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>899</v>
+        <v>901</v>
       </c>
       <c r="C38" s="4">
-        <v>2538</v>
+        <v>2811</v>
       </c>
       <c r="D38" s="4">
         <v>5</v>
@@ -18991,10 +18968,10 @@
         <v>29</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="G38" s="4">
-        <v>35</v>
+        <v>10</v>
+      </c>
+      <c r="G38" s="5">
+        <v>104.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
@@ -19005,10 +18982,10 @@
         <v>901</v>
       </c>
       <c r="C39" s="4">
-        <v>2811</v>
+        <v>2820</v>
       </c>
       <c r="D39" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E39" s="3" t="s">
         <v>29</v>
@@ -19016,22 +18993,22 @@
       <c r="F39" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G39" s="5">
-        <v>104.5</v>
+      <c r="G39" s="4">
+        <v>205</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
       <c r="A40" s="3" t="s">
-        <v>900</v>
+        <v>902</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>901</v>
+        <v>903</v>
       </c>
       <c r="C40" s="4">
-        <v>2820</v>
+        <v>3722</v>
       </c>
       <c r="D40" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E40" s="3" t="s">
         <v>29</v>
@@ -19040,7 +19017,7 @@
         <v>10</v>
       </c>
       <c r="G40" s="4">
-        <v>205</v>
+        <v>66</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
@@ -19051,30 +19028,30 @@
         <v>903</v>
       </c>
       <c r="C41" s="4">
-        <v>3722</v>
+        <v>4050</v>
       </c>
       <c r="D41" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>10</v>
+        <v>158</v>
       </c>
       <c r="G41" s="4">
-        <v>66</v>
+        <v>128</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
       <c r="A42" s="3" t="s">
-        <v>902</v>
+        <v>904</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="C42" s="4">
-        <v>4050</v>
+        <v>415</v>
       </c>
       <c r="D42" s="4">
         <v>10</v>
@@ -19083,21 +19060,21 @@
         <v>29</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>158</v>
+        <v>10</v>
       </c>
       <c r="G42" s="4">
-        <v>128</v>
+        <v>105</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
       <c r="A43" s="3" t="s">
-        <v>904</v>
+        <v>906</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>905</v>
+        <v>907</v>
       </c>
       <c r="C43" s="4">
-        <v>415</v>
+        <v>93</v>
       </c>
       <c r="D43" s="4">
         <v>10</v>
@@ -19109,30 +19086,30 @@
         <v>10</v>
       </c>
       <c r="G43" s="4">
-        <v>105</v>
+        <v>90</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
       <c r="A44" s="3" t="s">
-        <v>906</v>
+        <v>908</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>907</v>
+        <v>909</v>
       </c>
       <c r="C44" s="4">
-        <v>93</v>
+        <v>261</v>
       </c>
       <c r="D44" s="4">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E44" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>10</v>
+        <v>158</v>
       </c>
       <c r="G44" s="4">
-        <v>90</v>
+        <v>83</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
@@ -19143,42 +19120,42 @@
         <v>909</v>
       </c>
       <c r="C45" s="4">
-        <v>261</v>
+        <v>2475</v>
       </c>
       <c r="D45" s="4">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E45" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="G45" s="4">
-        <v>83</v>
+        <v>10</v>
+      </c>
+      <c r="G45" s="5">
+        <v>18.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
       <c r="A46" s="3" t="s">
-        <v>908</v>
+        <v>910</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>909</v>
+        <v>911</v>
       </c>
       <c r="C46" s="4">
-        <v>2475</v>
+        <v>92</v>
       </c>
       <c r="D46" s="4">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E46" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G46" s="5">
-        <v>18.5</v>
+        <v>158</v>
+      </c>
+      <c r="G46" s="4">
+        <v>67</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
@@ -19189,42 +19166,42 @@
         <v>911</v>
       </c>
       <c r="C47" s="4">
-        <v>92</v>
+        <v>2476</v>
       </c>
       <c r="D47" s="4">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="E47" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="G47" s="4">
-        <v>67</v>
+        <v>10</v>
+      </c>
+      <c r="G47" s="5">
+        <v>11.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
       <c r="A48" s="3" t="s">
-        <v>910</v>
+        <v>912</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>911</v>
+        <v>913</v>
       </c>
       <c r="C48" s="4">
-        <v>2476</v>
+        <v>18</v>
       </c>
       <c r="D48" s="4">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="E48" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G48" s="5">
-        <v>11.5</v>
+        <v>158</v>
+      </c>
+      <c r="G48" s="4">
+        <v>96</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
@@ -19235,42 +19212,42 @@
         <v>913</v>
       </c>
       <c r="C49" s="4">
-        <v>18</v>
+        <v>2477</v>
       </c>
       <c r="D49" s="4">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E49" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>158</v>
+        <v>10</v>
       </c>
       <c r="G49" s="4">
-        <v>96</v>
+        <v>22.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
       <c r="A50" s="3" t="s">
-        <v>912</v>
+        <v>914</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>913</v>
+        <v>915</v>
       </c>
       <c r="C50" s="4">
-        <v>2477</v>
+        <v>4164</v>
       </c>
       <c r="D50" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E50" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>10</v>
+        <v>158</v>
       </c>
       <c r="G50" s="4">
-        <v>22.5</v>
+        <v>180</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75">
@@ -19281,42 +19258,42 @@
         <v>915</v>
       </c>
       <c r="C51" s="4">
-        <v>4164</v>
+        <v>3706</v>
       </c>
       <c r="D51" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>158</v>
+        <v>10</v>
       </c>
       <c r="G51" s="4">
-        <v>170</v>
+        <v>92</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75">
       <c r="A52" s="3" t="s">
-        <v>914</v>
+        <v>916</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>915</v>
+        <v>917</v>
       </c>
       <c r="C52" s="4">
-        <v>3706</v>
+        <v>19</v>
       </c>
       <c r="D52" s="4">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E52" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>10</v>
+        <v>158</v>
       </c>
       <c r="G52" s="4">
-        <v>88</v>
+        <v>168</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75">
@@ -19327,19 +19304,19 @@
         <v>917</v>
       </c>
       <c r="C53" s="4">
-        <v>19</v>
+        <v>2246</v>
       </c>
       <c r="D53" s="4">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>29</v>
+        <v>344</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>158</v>
+        <v>49</v>
       </c>
       <c r="G53" s="4">
-        <v>168</v>
+        <v>192</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75">
@@ -19350,42 +19327,42 @@
         <v>917</v>
       </c>
       <c r="C54" s="4">
-        <v>2246</v>
+        <v>575</v>
       </c>
       <c r="D54" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>344</v>
+        <v>29</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="G54" s="4">
-        <v>192</v>
+        <v>48</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75">
       <c r="A55" s="3" t="s">
-        <v>916</v>
+        <v>918</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>917</v>
+        <v>919</v>
       </c>
       <c r="C55" s="4">
-        <v>575</v>
+        <v>221</v>
       </c>
       <c r="D55" s="4">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E55" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>10</v>
+        <v>158</v>
       </c>
       <c r="G55" s="4">
-        <v>48</v>
+        <v>300</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75">
@@ -19396,19 +19373,19 @@
         <v>919</v>
       </c>
       <c r="C56" s="4">
-        <v>221</v>
+        <v>258</v>
       </c>
       <c r="D56" s="4">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>29</v>
+        <v>344</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>158</v>
+        <v>49</v>
       </c>
       <c r="G56" s="4">
-        <v>300</v>
+        <v>324</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75">
@@ -19419,30 +19396,30 @@
         <v>919</v>
       </c>
       <c r="C57" s="4">
-        <v>258</v>
+        <v>20</v>
       </c>
       <c r="D57" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>344</v>
+        <v>29</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="G57" s="4">
-        <v>324</v>
+        <v>77</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75">
       <c r="A58" s="3" t="s">
-        <v>918</v>
+        <v>920</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>919</v>
+        <v>921</v>
       </c>
       <c r="C58" s="4">
-        <v>20</v>
+        <v>2520</v>
       </c>
       <c r="D58" s="4">
         <v>5</v>
@@ -19454,7 +19431,7 @@
         <v>10</v>
       </c>
       <c r="G58" s="4">
-        <v>77</v>
+        <v>29</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75">
@@ -19465,30 +19442,30 @@
         <v>921</v>
       </c>
       <c r="C59" s="4">
-        <v>2520</v>
+        <v>4089</v>
       </c>
       <c r="D59" s="4">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E59" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>10</v>
+        <v>158</v>
       </c>
       <c r="G59" s="4">
-        <v>29</v>
+        <v>130</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75">
       <c r="A60" s="3" t="s">
-        <v>920</v>
+        <v>922</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>921</v>
+        <v>923</v>
       </c>
       <c r="C60" s="4">
-        <v>4089</v>
+        <v>21</v>
       </c>
       <c r="D60" s="4">
         <v>25</v>
@@ -19500,18 +19477,18 @@
         <v>158</v>
       </c>
       <c r="G60" s="4">
-        <v>130</v>
+        <v>117</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75">
       <c r="A61" s="3" t="s">
-        <v>922</v>
+        <v>924</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>923</v>
+        <v>925</v>
       </c>
       <c r="C61" s="4">
-        <v>21</v>
+        <v>262</v>
       </c>
       <c r="D61" s="4">
         <v>25</v>
@@ -19523,7 +19500,7 @@
         <v>158</v>
       </c>
       <c r="G61" s="4">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18.75">
@@ -19534,42 +19511,42 @@
         <v>925</v>
       </c>
       <c r="C62" s="4">
-        <v>262</v>
+        <v>2513</v>
       </c>
       <c r="D62" s="4">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E62" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>158</v>
+        <v>10</v>
       </c>
       <c r="G62" s="4">
-        <v>119</v>
+        <v>26</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18.75">
       <c r="A63" s="3" t="s">
-        <v>924</v>
+        <v>926</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>925</v>
+        <v>927</v>
       </c>
       <c r="C63" s="4">
-        <v>2513</v>
+        <v>16</v>
       </c>
       <c r="D63" s="4">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E63" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>10</v>
+        <v>158</v>
       </c>
       <c r="G63" s="4">
-        <v>26</v>
+        <v>180</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18.75">
@@ -19580,65 +19557,65 @@
         <v>927</v>
       </c>
       <c r="C64" s="4">
-        <v>16</v>
+        <v>3114</v>
       </c>
       <c r="D64" s="4">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E64" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>158</v>
+        <v>10</v>
       </c>
       <c r="G64" s="4">
-        <v>180</v>
+        <v>38</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18.75">
       <c r="A65" s="3" t="s">
-        <v>926</v>
+        <v>928</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>927</v>
+        <v>929</v>
       </c>
       <c r="C65" s="4">
-        <v>3114</v>
+        <v>4086</v>
       </c>
       <c r="D65" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="G65" s="4">
-        <v>38</v>
+        <v>170</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75">
       <c r="A66" s="3" t="s">
-        <v>928</v>
+        <v>930</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>929</v>
+        <v>931</v>
       </c>
       <c r="C66" s="4">
-        <v>4086</v>
+        <v>15</v>
       </c>
       <c r="D66" s="4">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>49</v>
+        <v>158</v>
       </c>
       <c r="G66" s="4">
-        <v>170</v>
+        <v>190</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75">
@@ -19649,42 +19626,42 @@
         <v>931</v>
       </c>
       <c r="C67" s="4">
-        <v>15</v>
+        <v>3115</v>
       </c>
       <c r="D67" s="4">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E67" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>158</v>
+        <v>10</v>
       </c>
       <c r="G67" s="4">
-        <v>190</v>
+        <v>40</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75">
       <c r="A68" s="3" t="s">
-        <v>930</v>
+        <v>932</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>931</v>
+        <v>933</v>
       </c>
       <c r="C68" s="4">
-        <v>3115</v>
+        <v>4165</v>
       </c>
       <c r="D68" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E68" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>10</v>
+        <v>158</v>
       </c>
       <c r="G68" s="4">
-        <v>40</v>
+        <v>280</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75">
@@ -19695,42 +19672,42 @@
         <v>933</v>
       </c>
       <c r="C69" s="4">
-        <v>4165</v>
+        <v>4100</v>
       </c>
       <c r="D69" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E69" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>158</v>
+        <v>10</v>
       </c>
       <c r="G69" s="4">
-        <v>240</v>
+        <v>143.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18.75">
       <c r="A70" s="3" t="s">
-        <v>932</v>
+        <v>934</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>933</v>
+        <v>935</v>
       </c>
       <c r="C70" s="4">
-        <v>4100</v>
+        <v>4280</v>
       </c>
       <c r="D70" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E70" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>10</v>
+        <v>158</v>
       </c>
       <c r="G70" s="4">
-        <v>123.5</v>
+        <v>360</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18.75">
@@ -19741,10 +19718,10 @@
         <v>935</v>
       </c>
       <c r="C71" s="4">
-        <v>4280</v>
+        <v>4281</v>
       </c>
       <c r="D71" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E71" s="3" t="s">
         <v>29</v>
@@ -19753,29 +19730,6 @@
         <v>158</v>
       </c>
       <c r="G71" s="4">
-        <v>360</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18.75">
-      <c r="A72" s="3" t="s">
-        <v>934</v>
-      </c>
-      <c r="B72" s="3" t="s">
-        <v>935</v>
-      </c>
-      <c r="C72" s="4">
-        <v>4281</v>
-      </c>
-      <c r="D72" s="4">
-        <v>5</v>
-      </c>
-      <c r="E72" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F72" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="G72" s="4">
         <v>183.5</v>
       </c>
     </row>
@@ -19890,7 +19844,7 @@
         <v>158</v>
       </c>
       <c r="G4" s="4">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
@@ -19913,7 +19867,7 @@
         <v>10</v>
       </c>
       <c r="G5" s="4">
-        <v>24.5</v>
+        <v>24</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
@@ -20304,7 +20258,7 @@
         <v>158</v>
       </c>
       <c r="G22" s="4">
-        <v>485</v>
+        <v>495</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="19.5">
@@ -20327,7 +20281,7 @@
         <v>10</v>
       </c>
       <c r="G23" s="4">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="19.5">
@@ -20350,7 +20304,7 @@
         <v>10</v>
       </c>
       <c r="G24" s="4">
-        <v>485</v>
+        <v>495</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="19.5">
@@ -20373,7 +20327,7 @@
         <v>158</v>
       </c>
       <c r="G25" s="4">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="19.5">
@@ -20396,7 +20350,7 @@
         <v>158</v>
       </c>
       <c r="G26" s="4">
-        <v>485</v>
+        <v>495</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="19.5">
@@ -20419,7 +20373,7 @@
         <v>10</v>
       </c>
       <c r="G27" s="4">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="19.5">
@@ -20442,7 +20396,7 @@
         <v>158</v>
       </c>
       <c r="G28" s="4">
-        <v>485</v>
+        <v>495</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="19.5">
@@ -20465,7 +20419,7 @@
         <v>10</v>
       </c>
       <c r="G29" s="4">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="19.5">
@@ -21109,7 +21063,7 @@
         <v>158</v>
       </c>
       <c r="G57" s="4">
-        <v>330</v>
+        <v>350</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="19.5">
@@ -21132,7 +21086,7 @@
         <v>158</v>
       </c>
       <c r="G58" s="4">
-        <v>165</v>
+        <v>175</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="19.5">
@@ -21155,7 +21109,7 @@
         <v>10</v>
       </c>
       <c r="G59" s="4">
-        <v>30.5</v>
+        <v>32</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="19.5">
@@ -21546,7 +21500,7 @@
         <v>158</v>
       </c>
       <c r="G76" s="5">
-        <v>179</v>
+        <v>187.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18.75">
@@ -21569,7 +21523,7 @@
         <v>158</v>
       </c>
       <c r="G77" s="4">
-        <v>358</v>
+        <v>375</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18.75">
@@ -21592,7 +21546,7 @@
         <v>10</v>
       </c>
       <c r="G78" s="5">
-        <v>42.5</v>
+        <v>43.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18.75">
@@ -21868,7 +21822,7 @@
         <v>158</v>
       </c>
       <c r="G90" s="4">
-        <v>105</v>
+        <v>114</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18.75">
@@ -21891,7 +21845,7 @@
         <v>158</v>
       </c>
       <c r="G91" s="4">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18.75">
@@ -22028,7 +21982,7 @@
         <v>158</v>
       </c>
       <c r="G2" s="4">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
@@ -22376,7 +22330,7 @@
         <v>45</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="3" t="s">
         <v>391</v>
       </c>
@@ -22947,7 +22901,7 @@
         <v>158</v>
       </c>
       <c r="G2" s="4">
-        <v>412.5</v>
+        <v>475</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
@@ -22970,7 +22924,7 @@
         <v>10</v>
       </c>
       <c r="G3" s="4">
-        <v>51</v>
+        <v>59</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
@@ -23361,7 +23315,7 @@
         <v>158</v>
       </c>
       <c r="G20" s="4">
-        <v>1750</v>
+        <v>1875</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
@@ -23384,7 +23338,7 @@
         <v>10</v>
       </c>
       <c r="G21" s="4">
-        <v>350</v>
+        <v>375</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
@@ -23614,7 +23568,7 @@
         <v>158</v>
       </c>
       <c r="G31" s="5">
-        <v>73</v>
+        <v>77.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="19.5">
@@ -23637,7 +23591,7 @@
         <v>158</v>
       </c>
       <c r="G32" s="4">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="19.5">
@@ -24925,7 +24879,7 @@
         <v>158</v>
       </c>
       <c r="G88" s="4">
-        <v>182</v>
+        <v>202</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18.75">
@@ -24948,7 +24902,7 @@
         <v>10</v>
       </c>
       <c r="G89" s="5">
-        <v>38.5</v>
+        <v>43.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18.75">

</xml_diff>

<commit_message>
Atulizando demais valores 19/10
</commit_message>
<xml_diff>
--- a/data/ProdutosFomatodos.xlsx
+++ b/data/ProdutosFomatodos.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3771" uniqueCount="1147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3772" uniqueCount="1148">
   <si>
     <t>produto_grupo</t>
   </si>
@@ -2044,6 +2044,9 @@
   </si>
   <si>
     <t>PAINÇO</t>
+  </si>
+  <si>
+    <t>27.50</t>
   </si>
   <si>
     <t>pepita-de-girassol</t>
@@ -5797,16 +5800,16 @@
       <c r="F22" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G22" s="4">
-        <v>23</v>
+      <c r="G22" s="4" t="s">
+        <v>672</v>
       </c>
     </row>
     <row r="23" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="C23" s="4">
         <v>3417</v>
@@ -5826,10 +5829,10 @@
     </row>
     <row r="24" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="C24" s="4">
         <v>2716</v>
@@ -5849,10 +5852,10 @@
     </row>
     <row r="25" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="C25" s="4">
         <v>2478</v>
@@ -5872,10 +5875,10 @@
     </row>
     <row r="26" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="C26" s="4">
         <v>2606</v>
@@ -5895,10 +5898,10 @@
     </row>
     <row r="27" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="C27" s="4">
         <v>2338</v>
@@ -5918,10 +5921,10 @@
     </row>
     <row r="28" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="C28" s="4">
         <v>2425</v>
@@ -5941,10 +5944,10 @@
     </row>
     <row r="29" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="C29" s="4">
         <v>2579</v>
@@ -5964,10 +5967,10 @@
     </row>
     <row r="30" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="C30" s="4">
         <v>2243</v>
@@ -6028,7 +6031,7 @@
         <v>10</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
     </row>
     <row r="33" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -6079,10 +6082,10 @@
     </row>
     <row r="35" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="C35" s="4">
         <v>3754</v>
@@ -6145,10 +6148,10 @@
     </row>
     <row r="2" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="C2" s="4">
         <v>4336</v>
@@ -6168,10 +6171,10 @@
     </row>
     <row r="3" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="C3" s="4">
         <v>2618</v>
@@ -6191,10 +6194,10 @@
     </row>
     <row r="4" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="C4" s="4">
         <v>2398</v>
@@ -6214,10 +6217,10 @@
     </row>
     <row r="5" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="C5" s="4">
         <v>2297</v>
@@ -6237,10 +6240,10 @@
     </row>
     <row r="6" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="C6" s="4">
         <v>3653</v>
@@ -6260,10 +6263,10 @@
     </row>
     <row r="7" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="C7" s="4">
         <v>2339</v>
@@ -6283,10 +6286,10 @@
     </row>
     <row r="8" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="C8" s="4">
         <v>2223</v>
@@ -6306,10 +6309,10 @@
     </row>
     <row r="9" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="C9" s="4">
         <v>3707</v>
@@ -6329,10 +6332,10 @@
     </row>
     <row r="10" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="C10" s="4">
         <v>4090</v>
@@ -6352,10 +6355,10 @@
     </row>
     <row r="11" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="C11" s="4">
         <v>4279</v>
@@ -6398,10 +6401,10 @@
     </row>
     <row r="13" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="C13" s="4">
         <v>3540</v>
@@ -6421,10 +6424,10 @@
     </row>
     <row r="14" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="C14" s="4">
         <v>3541</v>
@@ -6513,10 +6516,10 @@
     </row>
     <row r="18" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="C18" s="4">
         <v>4639</v>
@@ -6536,10 +6539,10 @@
     </row>
     <row r="19" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="C19" s="4">
         <v>2336</v>
@@ -6559,10 +6562,10 @@
     </row>
     <row r="20" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="C20" s="4">
         <v>2421</v>
@@ -6582,10 +6585,10 @@
     </row>
     <row r="21" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="C21" s="4">
         <v>2568</v>
@@ -6605,10 +6608,10 @@
     </row>
     <row r="22" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="C22" s="4">
         <v>3009</v>
@@ -6628,10 +6631,10 @@
     </row>
     <row r="23" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="C23" s="4">
         <v>2778</v>
@@ -6651,10 +6654,10 @@
     </row>
     <row r="24" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="C24" s="4">
         <v>3106</v>
@@ -6674,10 +6677,10 @@
     </row>
     <row r="25" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="C25" s="4">
         <v>3489</v>
@@ -6697,10 +6700,10 @@
     </row>
     <row r="26" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="C26" s="4">
         <v>3696</v>
@@ -6720,10 +6723,10 @@
     </row>
     <row r="27" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="C27" s="4">
         <v>2783</v>
@@ -6743,10 +6746,10 @@
     </row>
     <row r="28" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="C28" s="4">
         <v>3755</v>
@@ -6766,10 +6769,10 @@
     </row>
     <row r="29" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="C29" s="4">
         <v>3486</v>
@@ -6789,10 +6792,10 @@
     </row>
     <row r="30" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="C30" s="4">
         <v>3487</v>
@@ -6812,10 +6815,10 @@
     </row>
     <row r="31" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="C31" s="4">
         <v>4488</v>
@@ -6835,10 +6838,10 @@
     </row>
     <row r="32" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="C32" s="4">
         <v>4333</v>
@@ -6858,10 +6861,10 @@
     </row>
     <row r="33" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="C33" s="4">
         <v>4650</v>
@@ -6881,10 +6884,10 @@
     </row>
     <row r="34" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="C34" s="4">
         <v>4388</v>
@@ -6904,10 +6907,10 @@
     </row>
     <row r="35" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="C35" s="4">
         <v>4389</v>
@@ -6927,10 +6930,10 @@
     </row>
     <row r="36" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="C36" s="4">
         <v>3488</v>
@@ -6950,10 +6953,10 @@
     </row>
     <row r="37" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="C37" s="4">
         <v>3400</v>
@@ -6973,10 +6976,10 @@
     </row>
     <row r="38" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="C38" s="4">
         <v>2257</v>
@@ -6996,10 +6999,10 @@
     </row>
     <row r="39" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="C39" s="4">
         <v>565</v>
@@ -7019,10 +7022,10 @@
     </row>
     <row r="40" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="C40" s="4">
         <v>4474</v>
@@ -7042,10 +7045,10 @@
     </row>
     <row r="41" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="C41" s="4">
         <v>4473</v>
@@ -7065,10 +7068,10 @@
     </row>
     <row r="42" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="C42" s="4">
         <v>2657</v>
@@ -7088,10 +7091,10 @@
     </row>
     <row r="43" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="C43" s="4">
         <v>2658</v>
@@ -7134,10 +7137,10 @@
     </row>
     <row r="45" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="C45" s="4">
         <v>3537</v>
@@ -7157,10 +7160,10 @@
     </row>
     <row r="46" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="C46" s="4">
         <v>2732</v>
@@ -7180,10 +7183,10 @@
     </row>
     <row r="47" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="C47" s="4">
         <v>2733</v>
@@ -7203,10 +7206,10 @@
     </row>
     <row r="48" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="C48" s="4">
         <v>2584</v>
@@ -7226,10 +7229,10 @@
     </row>
     <row r="49" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="C49" s="4">
         <v>2677</v>
@@ -7249,10 +7252,10 @@
     </row>
     <row r="50" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="C50" s="4">
         <v>2495</v>
@@ -7272,10 +7275,10 @@
     </row>
     <row r="51" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="C51" s="4">
         <v>2678</v>
@@ -7295,10 +7298,10 @@
     </row>
     <row r="52" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="C52" s="4">
         <v>4498</v>
@@ -7318,10 +7321,10 @@
     </row>
     <row r="53" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="C53" s="4">
         <v>4253</v>
@@ -7341,10 +7344,10 @@
     </row>
     <row r="54" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="C54" s="4">
         <v>4500</v>
@@ -7364,10 +7367,10 @@
     </row>
     <row r="55" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="C55" s="4">
         <v>4249</v>
@@ -7387,10 +7390,10 @@
     </row>
     <row r="56" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="C56" s="4">
         <v>3724</v>
@@ -7410,10 +7413,10 @@
     </row>
     <row r="57" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="C57" s="4">
         <v>3736</v>
@@ -7433,10 +7436,10 @@
     </row>
     <row r="58" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="C58" s="4">
         <v>4499</v>
@@ -7456,10 +7459,10 @@
     </row>
     <row r="59" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="C59" s="4">
         <v>3536</v>
@@ -7479,10 +7482,10 @@
     </row>
     <row r="60" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="C60" s="4">
         <v>2494</v>
@@ -7502,10 +7505,10 @@
     </row>
     <row r="61" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="C61" s="4">
         <v>2679</v>
@@ -7525,10 +7528,10 @@
     </row>
     <row r="62" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="C62" s="4">
         <v>4497</v>
@@ -7548,10 +7551,10 @@
     </row>
     <row r="63" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="C63" s="4">
         <v>2493</v>
@@ -7571,10 +7574,10 @@
     </row>
     <row r="64" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="C64" s="4">
         <v>3535</v>
@@ -7594,10 +7597,10 @@
     </row>
     <row r="65" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="C65" s="4">
         <v>2498</v>
@@ -7617,10 +7620,10 @@
     </row>
     <row r="66" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="C66" s="4">
         <v>2806</v>
@@ -7640,10 +7643,10 @@
     </row>
     <row r="67" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="C67" s="4">
         <v>2807</v>
@@ -7663,10 +7666,10 @@
     </row>
     <row r="68" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="C68" s="4">
         <v>4556</v>
@@ -7686,10 +7689,10 @@
     </row>
     <row r="69" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="C69" s="4">
         <v>4557</v>
@@ -7709,10 +7712,10 @@
     </row>
     <row r="70" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="C70" s="4">
         <v>4018</v>
@@ -7732,10 +7735,10 @@
     </row>
     <row r="71" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="C71" s="4">
         <v>2652</v>
@@ -7755,10 +7758,10 @@
     </row>
     <row r="72" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="C72" s="4">
         <v>4049</v>
@@ -7778,10 +7781,10 @@
     </row>
     <row r="73" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="C73" s="4">
         <v>3737</v>
@@ -7801,10 +7804,10 @@
     </row>
     <row r="74" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="C74" s="4">
         <v>4301</v>
@@ -7824,10 +7827,10 @@
     </row>
     <row r="75" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="C75" s="4">
         <v>4334</v>
@@ -7847,10 +7850,10 @@
     </row>
     <row r="76" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>766</v>
+        <v>767</v>
       </c>
       <c r="C76" s="4">
         <v>195</v>
@@ -7870,10 +7873,10 @@
     </row>
     <row r="77" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>766</v>
+        <v>767</v>
       </c>
       <c r="C77" s="4">
         <v>54</v>
@@ -7893,10 +7896,10 @@
     </row>
     <row r="78" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="C78" s="4">
         <v>63</v>
@@ -7916,10 +7919,10 @@
     </row>
     <row r="79" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="C79" s="4">
         <v>2483</v>
@@ -7939,10 +7942,10 @@
     </row>
     <row r="80" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="C80" s="4">
         <v>2974</v>
@@ -7962,10 +7965,10 @@
     </row>
     <row r="81" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="C81" s="4">
         <v>2831</v>
@@ -7985,10 +7988,10 @@
     </row>
     <row r="82" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="C82" s="4">
         <v>4137</v>
@@ -8008,10 +8011,10 @@
     </row>
     <row r="83" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>774</v>
+        <v>775</v>
       </c>
       <c r="C83" s="4">
         <v>4380</v>
@@ -8031,10 +8034,10 @@
     </row>
     <row r="84" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
-        <v>775</v>
+        <v>776</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="C84" s="4">
         <v>4566</v>
@@ -8054,10 +8057,10 @@
     </row>
     <row r="85" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="C85" s="4">
         <v>4567</v>
@@ -8077,10 +8080,10 @@
     </row>
     <row r="86" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
-        <v>779</v>
+        <v>780</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="C86" s="4">
         <v>4204</v>
@@ -8100,10 +8103,10 @@
     </row>
     <row r="87" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
-        <v>779</v>
+        <v>780</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="C87" s="4">
         <v>4205</v>
@@ -8123,10 +8126,10 @@
     </row>
     <row r="88" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>782</v>
+        <v>783</v>
       </c>
       <c r="C88" s="4">
         <v>4378</v>
@@ -8146,10 +8149,10 @@
     </row>
     <row r="89" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>782</v>
+        <v>783</v>
       </c>
       <c r="C89" s="4">
         <v>4379</v>
@@ -8169,10 +8172,10 @@
     </row>
     <row r="90" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>784</v>
+        <v>785</v>
       </c>
       <c r="C90" s="4">
         <v>3524</v>
@@ -8184,7 +8187,7 @@
         <v>9</v>
       </c>
       <c r="F90" s="3" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="G90" s="4">
         <v>350</v>
@@ -8192,10 +8195,10 @@
     </row>
     <row r="91" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>784</v>
+        <v>785</v>
       </c>
       <c r="C91" s="4">
         <v>3523</v>
@@ -8207,7 +8210,7 @@
         <v>9</v>
       </c>
       <c r="F91" s="3" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="G91" s="4">
         <v>72</v>
@@ -8215,10 +8218,10 @@
     </row>
     <row r="92" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>787</v>
+        <v>788</v>
       </c>
       <c r="C92" s="4">
         <v>3521</v>
@@ -8227,7 +8230,7 @@
         <v>16</v>
       </c>
       <c r="E92" s="3" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="F92" s="3" t="s">
         <v>28</v>
@@ -8238,10 +8241,10 @@
     </row>
     <row r="93" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>787</v>
+        <v>788</v>
       </c>
       <c r="C93" s="4">
         <v>3522</v>
@@ -8261,10 +8264,10 @@
     </row>
     <row r="94" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="C94" s="4">
         <v>64</v>
@@ -8284,10 +8287,10 @@
     </row>
     <row r="95" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="C95" s="4">
         <v>90</v>
@@ -8307,10 +8310,10 @@
     </row>
     <row r="96" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="C96" s="4">
         <v>3637</v>
@@ -8325,15 +8328,15 @@
         <v>10</v>
       </c>
       <c r="G96" s="4" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
     </row>
     <row r="97" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="C97" s="4">
         <v>2805</v>
@@ -8353,10 +8356,10 @@
     </row>
     <row r="98" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="C98" s="4">
         <v>2427</v>
@@ -8376,10 +8379,10 @@
     </row>
     <row r="99" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
-        <v>796</v>
+        <v>797</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="C99" s="4">
         <v>3437</v>
@@ -8399,10 +8402,10 @@
     </row>
     <row r="100" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" s="3" t="s">
-        <v>796</v>
+        <v>797</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="C100" s="4">
         <v>3396</v>
@@ -8422,10 +8425,10 @@
     </row>
     <row r="101" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="3" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="C101" s="4">
         <v>3395</v>
@@ -8434,7 +8437,7 @@
         <v>12</v>
       </c>
       <c r="E101" s="3" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="F101" s="3" t="s">
         <v>28</v>
@@ -8445,10 +8448,10 @@
     </row>
     <row r="102" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" s="3" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="C102" s="4">
         <v>3490</v>
@@ -8457,7 +8460,7 @@
         <v>12</v>
       </c>
       <c r="E102" s="3" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="F102" s="3" t="s">
         <v>28</v>
@@ -8468,10 +8471,10 @@
     </row>
     <row r="103" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>804</v>
+        <v>805</v>
       </c>
       <c r="C103" s="4">
         <v>458</v>
@@ -8480,7 +8483,7 @@
         <v>12</v>
       </c>
       <c r="E103" s="3" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="F103" s="3" t="s">
         <v>28</v>
@@ -8491,10 +8494,10 @@
     </row>
     <row r="104" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" s="3" t="s">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>807</v>
+        <v>808</v>
       </c>
       <c r="C104" s="4">
         <v>2641</v>
@@ -8503,7 +8506,7 @@
         <v>12</v>
       </c>
       <c r="E104" s="3" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="F104" s="3" t="s">
         <v>28</v>
@@ -8514,10 +8517,10 @@
     </row>
     <row r="105" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" s="3" t="s">
-        <v>808</v>
+        <v>809</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="C105" s="4">
         <v>4293</v>
@@ -8526,7 +8529,7 @@
         <v>12</v>
       </c>
       <c r="E105" s="3" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="F105" s="3" t="s">
         <v>28</v>
@@ -8537,10 +8540,10 @@
     </row>
     <row r="106" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" s="3" t="s">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="C106" s="4">
         <v>2396</v>
@@ -8560,10 +8563,10 @@
     </row>
     <row r="107" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" s="3" t="s">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="C107" s="4">
         <v>2426</v>
@@ -8583,10 +8586,10 @@
     </row>
     <row r="108" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" s="3" t="s">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="C108" s="4">
         <v>4335</v>
@@ -8606,10 +8609,10 @@
     </row>
     <row r="109" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" s="3" t="s">
-        <v>814</v>
+        <v>815</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>815</v>
+        <v>816</v>
       </c>
       <c r="C109" s="4">
         <v>4477</v>
@@ -8629,10 +8632,10 @@
     </row>
     <row r="110" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" s="3" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>817</v>
+        <v>818</v>
       </c>
       <c r="C110" s="4">
         <v>4479</v>
@@ -8652,10 +8655,10 @@
     </row>
     <row r="111" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" s="3" t="s">
-        <v>818</v>
+        <v>819</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>819</v>
+        <v>820</v>
       </c>
       <c r="C111" s="4">
         <v>4478</v>
@@ -8675,10 +8678,10 @@
     </row>
     <row r="112" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" s="3" t="s">
-        <v>820</v>
+        <v>821</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>821</v>
+        <v>822</v>
       </c>
       <c r="C112" s="4">
         <v>2646</v>
@@ -8687,7 +8690,7 @@
         <v>12</v>
       </c>
       <c r="E112" s="3" t="s">
-        <v>822</v>
+        <v>823</v>
       </c>
       <c r="F112" s="3" t="s">
         <v>273</v>
@@ -8698,10 +8701,10 @@
     </row>
     <row r="113" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" s="3" t="s">
-        <v>820</v>
+        <v>821</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>821</v>
+        <v>822</v>
       </c>
       <c r="C113" s="4">
         <v>2645</v>
@@ -8710,7 +8713,7 @@
         <v>6</v>
       </c>
       <c r="E113" s="3" t="s">
-        <v>823</v>
+        <v>824</v>
       </c>
       <c r="F113" s="3" t="s">
         <v>273</v>
@@ -8721,10 +8724,10 @@
     </row>
     <row r="114" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" s="3" t="s">
-        <v>820</v>
+        <v>821</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>821</v>
+        <v>822</v>
       </c>
       <c r="C114" s="4">
         <v>2638</v>
@@ -8733,7 +8736,7 @@
         <v>9</v>
       </c>
       <c r="E114" s="3" t="s">
-        <v>824</v>
+        <v>825</v>
       </c>
       <c r="F114" s="3" t="s">
         <v>273</v>
@@ -8744,10 +8747,10 @@
     </row>
     <row r="115" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" s="3" t="s">
-        <v>825</v>
+        <v>826</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>826</v>
+        <v>827</v>
       </c>
       <c r="C115" s="4">
         <v>4294</v>
@@ -8756,7 +8759,7 @@
         <v>18</v>
       </c>
       <c r="E115" s="3" t="s">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="F115" s="3" t="s">
         <v>273</v>
@@ -8767,10 +8770,10 @@
     </row>
     <row r="116" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" s="3" t="s">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="C116" s="4">
         <v>4314</v>
@@ -8790,10 +8793,10 @@
     </row>
     <row r="117" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117" s="3" t="s">
-        <v>830</v>
+        <v>831</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="C117" s="4">
         <v>4315</v>
@@ -8802,7 +8805,7 @@
         <v>15</v>
       </c>
       <c r="E117" s="3" t="s">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="F117" s="3" t="s">
         <v>28</v>
@@ -8856,10 +8859,10 @@
     </row>
     <row r="2" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="C2" s="4">
         <v>3402</v>
@@ -8868,7 +8871,7 @@
         <v>6</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>273</v>
@@ -8879,10 +8882,10 @@
     </row>
     <row r="3" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="C3" s="4">
         <v>3401</v>
@@ -8891,7 +8894,7 @@
         <v>6</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>273</v>
@@ -8902,10 +8905,10 @@
     </row>
     <row r="4" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="C4" s="4">
         <v>3403</v>
@@ -8914,7 +8917,7 @@
         <v>12</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>273</v>
@@ -8925,10 +8928,10 @@
     </row>
     <row r="5" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>839</v>
+        <v>840</v>
       </c>
       <c r="C5" s="4">
         <v>4032</v>
@@ -8937,7 +8940,7 @@
         <v>12</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>273</v>
@@ -8948,10 +8951,10 @@
     </row>
     <row r="6" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="C6" s="4">
         <v>4460</v>
@@ -8960,7 +8963,7 @@
         <v>12</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>273</v>
@@ -8971,10 +8974,10 @@
     </row>
     <row r="7" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="C7" s="4">
         <v>4260</v>
@@ -8983,7 +8986,7 @@
         <v>12</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>273</v>
@@ -8994,10 +8997,10 @@
     </row>
     <row r="8" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="C8" s="4">
         <v>2551</v>
@@ -9006,7 +9009,7 @@
         <v>12</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>273</v>
@@ -9017,10 +9020,10 @@
     </row>
     <row r="9" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>849</v>
+        <v>850</v>
       </c>
       <c r="C9" s="4">
         <v>2550</v>
@@ -9029,7 +9032,7 @@
         <v>6</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>273</v>
@@ -9040,10 +9043,10 @@
     </row>
     <row r="10" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="C10" s="4">
         <v>4383</v>
@@ -9052,7 +9055,7 @@
         <v>12</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>273</v>
@@ -9106,10 +9109,10 @@
     </row>
     <row r="2" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="C2" s="4">
         <v>3644</v>
@@ -9118,7 +9121,7 @@
         <v>12</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>273</v>
@@ -9129,10 +9132,10 @@
     </row>
     <row r="3" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="C3" s="4">
         <v>3644</v>
@@ -9141,7 +9144,7 @@
         <v>12</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>273</v>
@@ -9152,10 +9155,10 @@
     </row>
     <row r="4" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="C4" s="4">
         <v>3641</v>
@@ -9164,7 +9167,7 @@
         <v>24</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>273</v>
@@ -9175,10 +9178,10 @@
     </row>
     <row r="5" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="C5" s="4">
         <v>3645</v>
@@ -9187,7 +9190,7 @@
         <v>6</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>273</v>
@@ -9198,10 +9201,10 @@
     </row>
     <row r="6" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="C6" s="4">
         <v>3852</v>
@@ -9210,7 +9213,7 @@
         <v>12</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>11</v>
@@ -9221,10 +9224,10 @@
     </row>
     <row r="7" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="C7" s="4">
         <v>3647</v>
@@ -9233,7 +9236,7 @@
         <v>24</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>273</v>
@@ -9244,10 +9247,10 @@
     </row>
     <row r="8" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="C8" s="4">
         <v>3648</v>
@@ -9256,7 +9259,7 @@
         <v>6</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>858</v>
+        <v>859</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>273</v>
@@ -9310,10 +9313,10 @@
     </row>
     <row r="2" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="C2" s="4">
         <v>3056</v>
@@ -9328,15 +9331,15 @@
         <v>273</v>
       </c>
       <c r="G2" s="4">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="C3" s="4">
         <v>3083</v>
@@ -9351,15 +9354,15 @@
         <v>273</v>
       </c>
       <c r="G3" s="4">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="C4" s="4">
         <v>2264</v>
@@ -9374,15 +9377,15 @@
         <v>28</v>
       </c>
       <c r="G4" s="4">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="C5" s="4">
         <v>2355</v>
@@ -9397,15 +9400,15 @@
         <v>28</v>
       </c>
       <c r="G5" s="4">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="C6" s="4">
         <v>573</v>
@@ -9425,10 +9428,10 @@
     </row>
     <row r="7" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="C7" s="4">
         <v>572</v>
@@ -9448,10 +9451,10 @@
     </row>
     <row r="8" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="C8" s="4">
         <v>4411</v>
@@ -9471,10 +9474,10 @@
     </row>
     <row r="9" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="C9" s="4">
         <v>4410</v>
@@ -9537,10 +9540,10 @@
     </row>
     <row r="2" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="C2" s="4">
         <v>4044</v>
@@ -9549,7 +9552,7 @@
         <v>500</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
@@ -9560,10 +9563,10 @@
     </row>
     <row r="3" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="C3" s="4">
         <v>4672</v>
@@ -9572,7 +9575,7 @@
         <v>500</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>11</v>
@@ -9583,10 +9586,10 @@
     </row>
     <row r="4" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="C4" s="4">
         <v>4043</v>
@@ -9606,10 +9609,10 @@
     </row>
     <row r="5" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>873</v>
+        <v>874</v>
       </c>
       <c r="C5" s="4">
         <v>3531</v>
@@ -9629,10 +9632,10 @@
     </row>
     <row r="6" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>874</v>
+        <v>875</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="C6" s="4">
         <v>3974</v>
@@ -9652,10 +9655,10 @@
     </row>
     <row r="7" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="C7" s="4">
         <v>3530</v>
@@ -9675,10 +9678,10 @@
     </row>
     <row r="8" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="C8" s="4">
         <v>4282</v>
@@ -9698,10 +9701,10 @@
     </row>
     <row r="9" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>880</v>
+        <v>881</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>881</v>
+        <v>882</v>
       </c>
       <c r="C9" s="4">
         <v>3870</v>
@@ -9710,7 +9713,7 @@
         <v>500</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>11</v>
@@ -9721,10 +9724,10 @@
     </row>
     <row r="10" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="C10" s="4">
         <v>3701</v>
@@ -9733,7 +9736,7 @@
         <v>500</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>11</v>
@@ -9744,10 +9747,10 @@
     </row>
     <row r="11" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="C11" s="4">
         <v>3800</v>
@@ -9756,7 +9759,7 @@
         <v>500</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>11</v>
@@ -9767,10 +9770,10 @@
     </row>
     <row r="12" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>886</v>
+        <v>887</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="C12" s="4">
         <v>3725</v>
@@ -9779,7 +9782,7 @@
         <v>500</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>11</v>
@@ -9790,10 +9793,10 @@
     </row>
     <row r="13" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>889</v>
+        <v>890</v>
       </c>
       <c r="C13" s="4">
         <v>3871</v>
@@ -9802,7 +9805,7 @@
         <v>500</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>11</v>
@@ -9813,10 +9816,10 @@
     </row>
     <row r="14" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>890</v>
+        <v>891</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="C14" s="4">
         <v>2825</v>
@@ -9836,10 +9839,10 @@
     </row>
     <row r="15" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>892</v>
+        <v>893</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>893</v>
+        <v>894</v>
       </c>
       <c r="C15" s="4">
         <v>2828</v>
@@ -9859,10 +9862,10 @@
     </row>
     <row r="16" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>894</v>
+        <v>895</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
       <c r="C16" s="4">
         <v>2826</v>
@@ -9882,10 +9885,10 @@
     </row>
     <row r="17" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>896</v>
+        <v>897</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>897</v>
+        <v>898</v>
       </c>
       <c r="C17" s="4">
         <v>3058</v>
@@ -9905,10 +9908,10 @@
     </row>
     <row r="18" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>898</v>
+        <v>899</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>899</v>
+        <v>900</v>
       </c>
       <c r="C18" s="4">
         <v>3059</v>
@@ -9928,10 +9931,10 @@
     </row>
     <row r="19" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>900</v>
+        <v>901</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>901</v>
+        <v>902</v>
       </c>
       <c r="C19" s="4">
         <v>2829</v>
@@ -9951,10 +9954,10 @@
     </row>
     <row r="20" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>902</v>
+        <v>903</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>903</v>
+        <v>904</v>
       </c>
       <c r="C20" s="4">
         <v>4126</v>
@@ -9974,10 +9977,10 @@
     </row>
     <row r="21" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>905</v>
+        <v>906</v>
       </c>
       <c r="C21" s="4">
         <v>2827</v>
@@ -9997,10 +10000,10 @@
     </row>
     <row r="22" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>906</v>
+        <v>907</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>907</v>
+        <v>908</v>
       </c>
       <c r="C22" s="4">
         <v>3801</v>
@@ -10009,7 +10012,7 @@
         <v>500</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="F22" s="3" t="s">
         <v>11</v>
@@ -10020,10 +10023,10 @@
     </row>
     <row r="23" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>908</v>
+        <v>909</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>909</v>
+        <v>910</v>
       </c>
       <c r="C23" s="4">
         <v>3833</v>
@@ -10032,7 +10035,7 @@
         <v>500</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>11</v>
@@ -10043,10 +10046,10 @@
     </row>
     <row r="24" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>910</v>
+        <v>911</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>911</v>
+        <v>912</v>
       </c>
       <c r="C24" s="4">
         <v>3897</v>
@@ -10066,10 +10069,10 @@
     </row>
     <row r="25" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>912</v>
+        <v>913</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>913</v>
+        <v>914</v>
       </c>
       <c r="C25" s="4">
         <v>3764</v>
@@ -10178,10 +10181,10 @@
     </row>
     <row r="4" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>915</v>
+        <v>916</v>
       </c>
       <c r="C4" s="4">
         <v>3443</v>
@@ -10201,10 +10204,10 @@
     </row>
     <row r="5" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>915</v>
+        <v>916</v>
       </c>
       <c r="C5" s="4">
         <v>3019</v>
@@ -10224,10 +10227,10 @@
     </row>
     <row r="6" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>916</v>
+        <v>917</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>917</v>
+        <v>918</v>
       </c>
       <c r="C6" s="4">
         <v>4489</v>
@@ -10247,10 +10250,10 @@
     </row>
     <row r="7" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>916</v>
+        <v>917</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>917</v>
+        <v>918</v>
       </c>
       <c r="C7" s="4">
         <v>4490</v>
@@ -10270,10 +10273,10 @@
     </row>
     <row r="8" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>919</v>
+        <v>920</v>
       </c>
       <c r="C8" s="4">
         <v>3476</v>
@@ -10293,10 +10296,10 @@
     </row>
     <row r="9" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>919</v>
+        <v>920</v>
       </c>
       <c r="C9" s="4">
         <v>3477</v>
@@ -10316,10 +10319,10 @@
     </row>
     <row r="10" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>921</v>
+        <v>922</v>
       </c>
       <c r="C10" s="4">
         <v>4344</v>
@@ -10385,10 +10388,10 @@
     </row>
     <row r="13" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>922</v>
+        <v>923</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>923</v>
+        <v>924</v>
       </c>
       <c r="C13" s="4">
         <v>3719</v>
@@ -10408,10 +10411,10 @@
     </row>
     <row r="14" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>922</v>
+        <v>923</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>923</v>
+        <v>924</v>
       </c>
       <c r="C14" s="4">
         <v>3720</v>
@@ -10431,10 +10434,10 @@
     </row>
     <row r="15" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>924</v>
+        <v>925</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>925</v>
+        <v>926</v>
       </c>
       <c r="C15" s="4">
         <v>3765</v>
@@ -10454,10 +10457,10 @@
     </row>
     <row r="16" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>924</v>
+        <v>925</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>925</v>
+        <v>926</v>
       </c>
       <c r="C16" s="4">
         <v>3766</v>
@@ -10477,10 +10480,10 @@
     </row>
     <row r="17" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>926</v>
+        <v>927</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>927</v>
+        <v>928</v>
       </c>
       <c r="C17" s="4">
         <v>3126</v>
@@ -10500,10 +10503,10 @@
     </row>
     <row r="18" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>926</v>
+        <v>927</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>927</v>
+        <v>928</v>
       </c>
       <c r="C18" s="4">
         <v>3127</v>
@@ -10523,10 +10526,10 @@
     </row>
     <row r="19" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>928</v>
+        <v>929</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>929</v>
+        <v>930</v>
       </c>
       <c r="C19" s="4">
         <v>3435</v>
@@ -10546,10 +10549,10 @@
     </row>
     <row r="20" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>928</v>
+        <v>929</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>929</v>
+        <v>930</v>
       </c>
       <c r="C20" s="4">
         <v>3436</v>
@@ -10569,10 +10572,10 @@
     </row>
     <row r="21" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>930</v>
+        <v>931</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>931</v>
+        <v>932</v>
       </c>
       <c r="C21" s="4">
         <v>3128</v>
@@ -10592,10 +10595,10 @@
     </row>
     <row r="22" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>930</v>
+        <v>931</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>931</v>
+        <v>932</v>
       </c>
       <c r="C22" s="4">
         <v>3129</v>
@@ -10615,10 +10618,10 @@
     </row>
     <row r="23" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>932</v>
+        <v>933</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>933</v>
+        <v>934</v>
       </c>
       <c r="C23" s="4">
         <v>4158</v>
@@ -10638,10 +10641,10 @@
     </row>
     <row r="24" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>932</v>
+        <v>933</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>933</v>
+        <v>934</v>
       </c>
       <c r="C24" s="4">
         <v>4159</v>
@@ -10661,10 +10664,10 @@
     </row>
     <row r="25" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>934</v>
+        <v>935</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>935</v>
+        <v>936</v>
       </c>
       <c r="C25" s="4">
         <v>4561</v>
@@ -10684,10 +10687,10 @@
     </row>
     <row r="26" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>934</v>
+        <v>935</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>935</v>
+        <v>936</v>
       </c>
       <c r="C26" s="4">
         <v>4562</v>
@@ -10799,10 +10802,10 @@
     </row>
     <row r="31" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>936</v>
+        <v>937</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>937</v>
+        <v>938</v>
       </c>
       <c r="C31" s="4">
         <v>4346</v>
@@ -10822,10 +10825,10 @@
     </row>
     <row r="32" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>938</v>
+        <v>939</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="C32" s="4">
         <v>4345</v>
@@ -10845,10 +10848,10 @@
     </row>
     <row r="33" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>940</v>
+        <v>941</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>941</v>
+        <v>942</v>
       </c>
       <c r="C33" s="4">
         <v>4347</v>
@@ -10868,10 +10871,10 @@
     </row>
     <row r="34" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>942</v>
+        <v>943</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>943</v>
+        <v>944</v>
       </c>
       <c r="C34" s="4">
         <v>4446</v>
@@ -10891,10 +10894,10 @@
     </row>
     <row r="35" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>944</v>
+        <v>945</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>945</v>
+        <v>946</v>
       </c>
       <c r="C35" s="4">
         <v>4476</v>
@@ -10906,7 +10909,7 @@
         <v>9</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="G35" s="4">
         <v>33.5</v>
@@ -10914,10 +10917,10 @@
     </row>
     <row r="36" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>946</v>
+        <v>947</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>947</v>
+        <v>948</v>
       </c>
       <c r="C36" s="4">
         <v>4348</v>
@@ -10937,10 +10940,10 @@
     </row>
     <row r="37" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>948</v>
+        <v>949</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>949</v>
+        <v>950</v>
       </c>
       <c r="C37" s="4">
         <v>4456</v>
@@ -10960,10 +10963,10 @@
     </row>
     <row r="38" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="C38" s="4">
         <v>4051</v>
@@ -10983,10 +10986,10 @@
     </row>
     <row r="39" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="C39" s="4">
         <v>4408</v>
@@ -11006,10 +11009,10 @@
     </row>
     <row r="40" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>954</v>
+        <v>955</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>955</v>
+        <v>956</v>
       </c>
       <c r="C40" s="4">
         <v>4341</v>
@@ -11029,10 +11032,10 @@
     </row>
     <row r="41" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>956</v>
+        <v>957</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>957</v>
+        <v>958</v>
       </c>
       <c r="C41" s="4">
         <v>4265</v>
@@ -11052,10 +11055,10 @@
     </row>
     <row r="42" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>958</v>
+        <v>959</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>959</v>
+        <v>960</v>
       </c>
       <c r="C42" s="4">
         <v>4266</v>
@@ -11075,10 +11078,10 @@
     </row>
     <row r="43" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
       <c r="C43" s="4">
         <v>4269</v>
@@ -11098,10 +11101,10 @@
     </row>
     <row r="44" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>962</v>
+        <v>963</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>963</v>
+        <v>964</v>
       </c>
       <c r="C44" s="4">
         <v>4273</v>
@@ -11121,10 +11124,10 @@
     </row>
     <row r="45" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
       <c r="C45" s="4">
         <v>4405</v>
@@ -11144,10 +11147,10 @@
     </row>
     <row r="46" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>966</v>
+        <v>967</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>967</v>
+        <v>968</v>
       </c>
       <c r="C46" s="4">
         <v>4406</v>
@@ -11167,10 +11170,10 @@
     </row>
     <row r="47" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>969</v>
+        <v>970</v>
       </c>
       <c r="C47" s="4">
         <v>4267</v>
@@ -11190,10 +11193,10 @@
     </row>
     <row r="48" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>970</v>
+        <v>971</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>971</v>
+        <v>972</v>
       </c>
       <c r="C48" s="4">
         <v>4271</v>
@@ -11213,10 +11216,10 @@
     </row>
     <row r="49" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>972</v>
+        <v>973</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="C49" s="4">
         <v>4276</v>
@@ -11236,10 +11239,10 @@
     </row>
     <row r="50" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>974</v>
+        <v>975</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>975</v>
+        <v>976</v>
       </c>
       <c r="C50" s="4">
         <v>4342</v>
@@ -11259,10 +11262,10 @@
     </row>
     <row r="51" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
-        <v>976</v>
+        <v>977</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>977</v>
+        <v>978</v>
       </c>
       <c r="C51" s="4">
         <v>2505</v>
@@ -11282,10 +11285,10 @@
     </row>
     <row r="52" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
-        <v>978</v>
+        <v>979</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>979</v>
+        <v>980</v>
       </c>
       <c r="C52" s="4">
         <v>4398</v>
@@ -11305,10 +11308,10 @@
     </row>
     <row r="53" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
-        <v>980</v>
+        <v>981</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>981</v>
+        <v>982</v>
       </c>
       <c r="C53" s="4">
         <v>4270</v>
@@ -11328,10 +11331,10 @@
     </row>
     <row r="54" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>982</v>
+        <v>983</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>983</v>
+        <v>984</v>
       </c>
       <c r="C54" s="4">
         <v>4275</v>
@@ -11351,10 +11354,10 @@
     </row>
     <row r="55" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
-        <v>984</v>
+        <v>985</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>985</v>
+        <v>986</v>
       </c>
       <c r="C55" s="4">
         <v>4274</v>
@@ -11374,10 +11377,10 @@
     </row>
     <row r="56" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>986</v>
+        <v>987</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>987</v>
+        <v>988</v>
       </c>
       <c r="C56" s="4">
         <v>4399</v>
@@ -11397,10 +11400,10 @@
     </row>
     <row r="57" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
-        <v>988</v>
+        <v>989</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>989</v>
+        <v>990</v>
       </c>
       <c r="C57" s="4">
         <v>4404</v>
@@ -11420,10 +11423,10 @@
     </row>
     <row r="58" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
-        <v>990</v>
+        <v>991</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>991</v>
+        <v>992</v>
       </c>
       <c r="C58" s="4">
         <v>4262</v>
@@ -11443,10 +11446,10 @@
     </row>
     <row r="59" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
-        <v>992</v>
+        <v>993</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
       <c r="C59" s="4">
         <v>4263</v>
@@ -11466,10 +11469,10 @@
     </row>
     <row r="60" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
-        <v>994</v>
+        <v>995</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>995</v>
+        <v>996</v>
       </c>
       <c r="C60" s="4">
         <v>4264</v>
@@ -11489,10 +11492,10 @@
     </row>
     <row r="61" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
-        <v>996</v>
+        <v>997</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>997</v>
+        <v>998</v>
       </c>
       <c r="C61" s="4">
         <v>4407</v>
@@ -11512,10 +11515,10 @@
     </row>
     <row r="62" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
-        <v>998</v>
+        <v>999</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>999</v>
+        <v>1000</v>
       </c>
       <c r="C62" s="4">
         <v>4397</v>
@@ -11535,10 +11538,10 @@
     </row>
     <row r="63" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
-        <v>1000</v>
+        <v>1001</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>1001</v>
+        <v>1002</v>
       </c>
       <c r="C63" s="4">
         <v>4343</v>
@@ -11558,10 +11561,10 @@
     </row>
     <row r="64" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
-        <v>1002</v>
+        <v>1003</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>1003</v>
+        <v>1004</v>
       </c>
       <c r="C64" s="4">
         <v>4268</v>
@@ -11581,10 +11584,10 @@
     </row>
     <row r="65" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
-        <v>1004</v>
+        <v>1005</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>1005</v>
+        <v>1006</v>
       </c>
       <c r="C65" s="4">
         <v>2833</v>
@@ -11604,10 +11607,10 @@
     </row>
     <row r="66" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
-        <v>1004</v>
+        <v>1005</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>1005</v>
+        <v>1006</v>
       </c>
       <c r="C66" s="4">
         <v>3125</v>
@@ -11627,10 +11630,10 @@
     </row>
     <row r="67" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
-        <v>1006</v>
+        <v>1007</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>1007</v>
+        <v>1008</v>
       </c>
       <c r="C67" s="4">
         <v>3752</v>
@@ -11650,10 +11653,10 @@
     </row>
     <row r="68" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
-        <v>1006</v>
+        <v>1007</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>1007</v>
+        <v>1008</v>
       </c>
       <c r="C68" s="4">
         <v>3753</v>
@@ -11673,10 +11676,10 @@
     </row>
     <row r="69" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>1009</v>
+        <v>1010</v>
       </c>
       <c r="C69" s="4">
         <v>2511</v>
@@ -11696,10 +11699,10 @@
     </row>
     <row r="70" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
-        <v>1010</v>
+        <v>1011</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>1011</v>
+        <v>1012</v>
       </c>
       <c r="C70" s="4">
         <v>4311</v>
@@ -11719,10 +11722,10 @@
     </row>
     <row r="71" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
-        <v>1012</v>
+        <v>1013</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>1013</v>
+        <v>1014</v>
       </c>
       <c r="C71" s="4">
         <v>4046</v>
@@ -11742,10 +11745,10 @@
     </row>
     <row r="72" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
-        <v>1012</v>
+        <v>1013</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>1013</v>
+        <v>1014</v>
       </c>
       <c r="C72" s="4">
         <v>4047</v>
@@ -11765,10 +11768,10 @@
     </row>
     <row r="73" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
-        <v>1014</v>
+        <v>1015</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>1015</v>
+        <v>1016</v>
       </c>
       <c r="C73" s="4">
         <v>4312</v>
@@ -11788,10 +11791,10 @@
     </row>
     <row r="74" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
-        <v>1016</v>
+        <v>1017</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="C74" s="4">
         <v>4310</v>
@@ -11811,10 +11814,10 @@
     </row>
     <row r="75" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>1019</v>
+        <v>1020</v>
       </c>
       <c r="C75" s="4">
         <v>4074</v>
@@ -11823,7 +11826,7 @@
         <v>1</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>1020</v>
+        <v>1021</v>
       </c>
       <c r="F75" s="3" t="s">
         <v>11</v>
@@ -11834,10 +11837,10 @@
     </row>
     <row r="76" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
-        <v>1021</v>
+        <v>1022</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>1022</v>
+        <v>1023</v>
       </c>
       <c r="C76" s="4">
         <v>4076</v>
@@ -11846,10 +11849,10 @@
         <v>1</v>
       </c>
       <c r="E76" s="3" t="s">
-        <v>1023</v>
+        <v>1024</v>
       </c>
       <c r="F76" s="3" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="G76" s="4">
         <v>32.5</v>
@@ -11857,10 +11860,10 @@
     </row>
     <row r="77" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
-        <v>1025</v>
+        <v>1026</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>1026</v>
+        <v>1027</v>
       </c>
       <c r="C77" s="4">
         <v>4133</v>
@@ -11872,7 +11875,7 @@
         <v>426</v>
       </c>
       <c r="F77" s="3" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="G77" s="4">
         <v>72</v>
@@ -11880,10 +11883,10 @@
     </row>
     <row r="78" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="s">
-        <v>1027</v>
+        <v>1028</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>1028</v>
+        <v>1029</v>
       </c>
       <c r="C78" s="4">
         <v>3068</v>
@@ -11903,10 +11906,10 @@
     </row>
     <row r="79" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
-        <v>1027</v>
+        <v>1028</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>1028</v>
+        <v>1029</v>
       </c>
       <c r="C79" s="4">
         <v>3087</v>
@@ -11926,10 +11929,10 @@
     </row>
     <row r="80" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
-        <v>1029</v>
+        <v>1030</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>1030</v>
+        <v>1031</v>
       </c>
       <c r="C80" s="4">
         <v>4560</v>
@@ -11949,10 +11952,10 @@
     </row>
     <row r="81" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
-        <v>1031</v>
+        <v>1032</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
       <c r="C81" s="4">
         <v>4531</v>
@@ -11972,10 +11975,10 @@
     </row>
     <row r="82" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
-        <v>1031</v>
+        <v>1032</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
       <c r="C82" s="4">
         <v>4532</v>
@@ -11995,10 +11998,10 @@
     </row>
     <row r="83" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
-        <v>1033</v>
+        <v>1034</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="C83" s="4">
         <v>4559</v>
@@ -12018,10 +12021,10 @@
     </row>
     <row r="84" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
-        <v>1035</v>
+        <v>1036</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
       <c r="C84" s="4">
         <v>4493</v>
@@ -12041,10 +12044,10 @@
     </row>
     <row r="85" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
       <c r="C85" s="4">
         <v>4102</v>
@@ -12053,7 +12056,7 @@
         <v>10</v>
       </c>
       <c r="E85" s="3" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="F85" s="3" t="s">
         <v>11</v>
@@ -12064,10 +12067,10 @@
     </row>
     <row r="86" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
-        <v>1040</v>
+        <v>1041</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="C86" s="4">
         <v>4103</v>
@@ -12076,7 +12079,7 @@
         <v>10</v>
       </c>
       <c r="E86" s="3" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="F86" s="3" t="s">
         <v>273</v>
@@ -12087,10 +12090,10 @@
     </row>
     <row r="87" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
-        <v>1042</v>
+        <v>1043</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>1043</v>
+        <v>1044</v>
       </c>
       <c r="C87" s="4">
         <v>4547</v>
@@ -12099,7 +12102,7 @@
         <v>10</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="F87" s="3" t="s">
         <v>273</v>
@@ -12110,10 +12113,10 @@
     </row>
     <row r="88" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
-        <v>1044</v>
+        <v>1045</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>1045</v>
+        <v>1046</v>
       </c>
       <c r="C88" s="4">
         <v>4624</v>
@@ -12122,7 +12125,7 @@
         <v>21</v>
       </c>
       <c r="E88" s="3" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="F88" s="3" t="s">
         <v>11</v>
@@ -12133,10 +12136,10 @@
     </row>
     <row r="89" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="C89" s="4">
         <v>4627</v>
@@ -12145,7 +12148,7 @@
         <v>25</v>
       </c>
       <c r="E89" s="3" t="s">
-        <v>1049</v>
+        <v>1050</v>
       </c>
       <c r="F89" s="3" t="s">
         <v>11</v>
@@ -12156,10 +12159,10 @@
     </row>
     <row r="90" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>1051</v>
+        <v>1052</v>
       </c>
       <c r="C90" s="4">
         <v>4628</v>
@@ -12168,7 +12171,7 @@
         <v>15</v>
       </c>
       <c r="E90" s="3" t="s">
-        <v>1052</v>
+        <v>1053</v>
       </c>
       <c r="F90" s="3" t="s">
         <v>11</v>
@@ -12179,10 +12182,10 @@
     </row>
     <row r="91" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
-        <v>1053</v>
+        <v>1054</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>1054</v>
+        <v>1055</v>
       </c>
       <c r="C91" s="4">
         <v>4625</v>
@@ -12191,7 +12194,7 @@
         <v>21</v>
       </c>
       <c r="E91" s="3" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="F91" s="3" t="s">
         <v>11</v>
@@ -12202,10 +12205,10 @@
     </row>
     <row r="92" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
-        <v>1055</v>
+        <v>1056</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>1056</v>
+        <v>1057</v>
       </c>
       <c r="C92" s="4">
         <v>4626</v>
@@ -12214,7 +12217,7 @@
         <v>21</v>
       </c>
       <c r="E92" s="3" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="F92" s="3" t="s">
         <v>11</v>
@@ -12225,10 +12228,10 @@
     </row>
     <row r="93" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
-        <v>1057</v>
+        <v>1058</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>1058</v>
+        <v>1059</v>
       </c>
       <c r="C93" s="4">
         <v>4699</v>
@@ -12237,7 +12240,7 @@
         <v>50</v>
       </c>
       <c r="E93" s="3" t="s">
-        <v>1059</v>
+        <v>1060</v>
       </c>
       <c r="F93" s="3" t="s">
         <v>273</v>
@@ -12248,10 +12251,10 @@
     </row>
     <row r="94" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
-        <v>1060</v>
+        <v>1061</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="C94" s="4">
         <v>4643</v>
@@ -12260,10 +12263,10 @@
         <v>6</v>
       </c>
       <c r="E94" s="3" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="F94" s="3" t="s">
-        <v>1062</v>
+        <v>1063</v>
       </c>
       <c r="G94" s="4">
         <v>97.5</v>
@@ -12271,10 +12274,10 @@
     </row>
     <row r="95" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
-        <v>1063</v>
+        <v>1064</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>1064</v>
+        <v>1065</v>
       </c>
       <c r="C95" s="4">
         <v>4687</v>
@@ -12283,10 +12286,10 @@
         <v>6</v>
       </c>
       <c r="E95" s="3" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="F95" s="3" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="G95" s="4">
         <v>64</v>
@@ -12294,10 +12297,10 @@
     </row>
     <row r="96" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
-        <v>1065</v>
+        <v>1066</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="C96" s="4">
         <v>4644</v>
@@ -12306,10 +12309,10 @@
         <v>6</v>
       </c>
       <c r="E96" s="3" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="F96" s="3" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="G96" s="4">
         <v>57</v>
@@ -12317,10 +12320,10 @@
     </row>
     <row r="97" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
-        <v>1067</v>
+        <v>1068</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="C97" s="4">
         <v>4104</v>
@@ -12329,7 +12332,7 @@
         <v>10</v>
       </c>
       <c r="E97" s="3" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="F97" s="3" t="s">
         <v>273</v>
@@ -12340,10 +12343,10 @@
     </row>
     <row r="98" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
-        <v>1069</v>
+        <v>1070</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>1070</v>
+        <v>1071</v>
       </c>
       <c r="C98" s="4">
         <v>4101</v>
@@ -12352,7 +12355,7 @@
         <v>10</v>
       </c>
       <c r="E98" s="3" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="F98" s="3" t="s">
         <v>273</v>
@@ -12363,10 +12366,10 @@
     </row>
     <row r="99" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="C99" s="4">
         <v>4105</v>
@@ -12375,7 +12378,7 @@
         <v>10</v>
       </c>
       <c r="E99" s="3" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="F99" s="3" t="s">
         <v>273</v>
@@ -12386,10 +12389,10 @@
     </row>
     <row r="100" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" s="3" t="s">
-        <v>1073</v>
+        <v>1074</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>1074</v>
+        <v>1075</v>
       </c>
       <c r="C100" s="4">
         <v>3705</v>
@@ -12398,7 +12401,7 @@
         <v>12</v>
       </c>
       <c r="E100" s="3" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="F100" s="3" t="s">
         <v>273</v>
@@ -12409,10 +12412,10 @@
     </row>
     <row r="101" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="3" t="s">
-        <v>1076</v>
+        <v>1077</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>1077</v>
+        <v>1078</v>
       </c>
       <c r="C101" s="4">
         <v>3823</v>
@@ -12421,7 +12424,7 @@
         <v>10</v>
       </c>
       <c r="E101" s="3" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="F101" s="3" t="s">
         <v>28</v>
@@ -12432,10 +12435,10 @@
     </row>
     <row r="102" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" s="3" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>1079</v>
+        <v>1080</v>
       </c>
       <c r="C102" s="4">
         <v>4641</v>
@@ -12444,7 +12447,7 @@
         <v>6</v>
       </c>
       <c r="E102" s="3" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="F102" s="3" t="s">
         <v>11</v>
@@ -12455,10 +12458,10 @@
     </row>
     <row r="103" ht="19.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>1080</v>
+        <v>1081</v>
       </c>
       <c r="C103" s="4">
         <v>4583</v>
@@ -12467,7 +12470,7 @@
         <v>12</v>
       </c>
       <c r="E103" s="3" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="F103" s="3" t="s">
         <v>273</v>
@@ -12478,10 +12481,10 @@
     </row>
     <row r="104" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" s="3" t="s">
-        <v>1081</v>
+        <v>1082</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>1082</v>
+        <v>1083</v>
       </c>
       <c r="C104" s="4">
         <v>4308</v>
@@ -12490,7 +12493,7 @@
         <v>10</v>
       </c>
       <c r="E104" s="3" t="s">
-        <v>1083</v>
+        <v>1084</v>
       </c>
       <c r="F104" s="3" t="s">
         <v>11</v>
@@ -12501,10 +12504,10 @@
     </row>
     <row r="105" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" s="3" t="s">
-        <v>1084</v>
+        <v>1085</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>1085</v>
+        <v>1086</v>
       </c>
       <c r="C105" s="4">
         <v>4309</v>
@@ -12513,10 +12516,10 @@
         <v>10</v>
       </c>
       <c r="E105" s="3" t="s">
-        <v>1083</v>
+        <v>1084</v>
       </c>
       <c r="F105" s="3" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="G105" s="4">
         <v>68.5</v>
@@ -12524,10 +12527,10 @@
     </row>
     <row r="106" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" s="3" t="s">
-        <v>1086</v>
+        <v>1087</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="C106" s="4">
         <v>4635</v>
@@ -12539,7 +12542,7 @@
         <v>426</v>
       </c>
       <c r="F106" s="3" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="G106" s="4">
         <v>177</v>
@@ -12547,10 +12550,10 @@
     </row>
     <row r="107" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" s="3" t="s">
-        <v>1088</v>
+        <v>1089</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>1089</v>
+        <v>1090</v>
       </c>
       <c r="C107" s="4">
         <v>4412</v>
@@ -12562,7 +12565,7 @@
         <v>9</v>
       </c>
       <c r="F107" s="3" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="G107" s="4">
         <v>75.5</v>
@@ -12570,10 +12573,10 @@
     </row>
     <row r="108" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" s="3" t="s">
-        <v>1090</v>
+        <v>1091</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="C108" s="4">
         <v>4413</v>
@@ -12593,10 +12596,10 @@
     </row>
     <row r="109" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" s="3" t="s">
-        <v>1090</v>
+        <v>1091</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="C109" s="4">
         <v>4414</v>
@@ -12616,10 +12619,10 @@
     </row>
     <row r="110" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" s="3" t="s">
-        <v>1092</v>
+        <v>1093</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>1093</v>
+        <v>1094</v>
       </c>
       <c r="C110" s="4">
         <v>4415</v>
@@ -12639,10 +12642,10 @@
     </row>
     <row r="111" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" s="3" t="s">
-        <v>1092</v>
+        <v>1093</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>1093</v>
+        <v>1094</v>
       </c>
       <c r="C111" s="4">
         <v>4416</v>
@@ -12662,10 +12665,10 @@
     </row>
     <row r="112" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" s="3" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>1095</v>
+        <v>1096</v>
       </c>
       <c r="C112" s="4">
         <v>4475</v>
@@ -12674,7 +12677,7 @@
         <v>1</v>
       </c>
       <c r="E112" s="3" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="F112" s="3" t="s">
         <v>11</v>
@@ -12685,10 +12688,10 @@
     </row>
     <row r="113" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" s="3" t="s">
-        <v>1097</v>
+        <v>1098</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>1098</v>
+        <v>1099</v>
       </c>
       <c r="C113" s="4">
         <v>4354</v>
@@ -12697,10 +12700,10 @@
         <v>12</v>
       </c>
       <c r="E113" s="3" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="F113" s="3" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="G113" s="4">
         <v>79.5</v>
@@ -12708,10 +12711,10 @@
     </row>
     <row r="114" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" s="3" t="s">
-        <v>1099</v>
+        <v>1100</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="C114" s="4">
         <v>4445</v>
@@ -12720,7 +12723,7 @@
         <v>12</v>
       </c>
       <c r="E114" s="3" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="F114" s="3" t="s">
         <v>28</v>
@@ -12731,10 +12734,10 @@
     </row>
     <row r="115" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" s="3" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="C115" s="4">
         <v>4353</v>
@@ -12743,7 +12746,7 @@
         <v>12</v>
       </c>
       <c r="E115" s="3" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="F115" s="3" t="s">
         <v>28</v>
@@ -12754,10 +12757,10 @@
     </row>
     <row r="116" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" s="3" t="s">
-        <v>1103</v>
+        <v>1104</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>1104</v>
+        <v>1105</v>
       </c>
       <c r="C116" s="4">
         <v>4350</v>
@@ -12766,7 +12769,7 @@
         <v>12</v>
       </c>
       <c r="E116" s="3" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="F116" s="3" t="s">
         <v>28</v>
@@ -12777,10 +12780,10 @@
     </row>
     <row r="117" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117" s="3" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>1106</v>
+        <v>1107</v>
       </c>
       <c r="C117" s="4">
         <v>4352</v>
@@ -12789,7 +12792,7 @@
         <v>12</v>
       </c>
       <c r="E117" s="3" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="F117" s="3" t="s">
         <v>28</v>
@@ -12800,10 +12803,10 @@
     </row>
     <row r="118" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A118" s="3" t="s">
-        <v>1107</v>
+        <v>1108</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>1108</v>
+        <v>1109</v>
       </c>
       <c r="C118" s="4">
         <v>4349</v>
@@ -12812,7 +12815,7 @@
         <v>12</v>
       </c>
       <c r="E118" s="3" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="F118" s="3" t="s">
         <v>28</v>
@@ -12823,10 +12826,10 @@
     </row>
     <row r="119" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119" s="3" t="s">
-        <v>1109</v>
+        <v>1110</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="C119" s="4">
         <v>4351</v>
@@ -12835,7 +12838,7 @@
         <v>12</v>
       </c>
       <c r="E119" s="3" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="F119" s="3" t="s">
         <v>28</v>
@@ -12846,10 +12849,10 @@
     </row>
     <row r="120" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" s="3" t="s">
-        <v>1111</v>
+        <v>1112</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>1112</v>
+        <v>1113</v>
       </c>
       <c r="C120" s="4">
         <v>4581</v>
@@ -12858,7 +12861,7 @@
         <v>12</v>
       </c>
       <c r="E120" s="3" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="F120" s="3" t="s">
         <v>28</v>
@@ -12869,10 +12872,10 @@
     </row>
     <row r="121" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121" s="3" t="s">
-        <v>1113</v>
+        <v>1114</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>1114</v>
+        <v>1115</v>
       </c>
       <c r="C121" s="4">
         <v>4096</v>
@@ -12892,10 +12895,10 @@
     </row>
     <row r="122" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122" s="3" t="s">
-        <v>1115</v>
+        <v>1116</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>1116</v>
+        <v>1117</v>
       </c>
       <c r="C122" s="4">
         <v>4582</v>
@@ -12904,7 +12907,7 @@
         <v>30</v>
       </c>
       <c r="E122" s="3" t="s">
-        <v>1117</v>
+        <v>1118</v>
       </c>
       <c r="F122" s="3" t="s">
         <v>11</v>
@@ -12915,10 +12918,10 @@
     </row>
     <row r="123" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A123" s="3" t="s">
-        <v>1118</v>
+        <v>1119</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>1119</v>
+        <v>1120</v>
       </c>
       <c r="C123" s="4">
         <v>4123</v>
@@ -12927,7 +12930,7 @@
         <v>10</v>
       </c>
       <c r="E123" s="3" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="F123" s="3" t="s">
         <v>11</v>
@@ -12938,10 +12941,10 @@
     </row>
     <row r="124" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A124" s="3" t="s">
-        <v>1120</v>
+        <v>1121</v>
       </c>
       <c r="B124" s="3" t="s">
-        <v>1121</v>
+        <v>1122</v>
       </c>
       <c r="C124" s="4">
         <v>4306</v>
@@ -12950,10 +12953,10 @@
         <v>10</v>
       </c>
       <c r="E124" s="3" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="F124" s="3" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="G124" s="4">
         <v>81</v>
@@ -12961,10 +12964,10 @@
     </row>
     <row r="125" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A125" s="3" t="s">
-        <v>1122</v>
+        <v>1123</v>
       </c>
       <c r="B125" s="3" t="s">
-        <v>1123</v>
+        <v>1124</v>
       </c>
       <c r="C125" s="4">
         <v>4307</v>
@@ -12973,10 +12976,10 @@
         <v>10</v>
       </c>
       <c r="E125" s="3" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="F125" s="3" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="G125" s="4">
         <v>81</v>
@@ -12984,10 +12987,10 @@
     </row>
     <row r="126" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A126" s="3" t="s">
-        <v>1124</v>
+        <v>1125</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>1125</v>
+        <v>1126</v>
       </c>
       <c r="C126" s="4">
         <v>2659</v>
@@ -12996,7 +12999,7 @@
         <v>20</v>
       </c>
       <c r="E126" s="3" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="F126" s="3" t="s">
         <v>273</v>
@@ -13007,10 +13010,10 @@
     </row>
     <row r="127" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A127" s="3" t="s">
-        <v>1124</v>
+        <v>1125</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>1125</v>
+        <v>1126</v>
       </c>
       <c r="C127" s="4">
         <v>2621</v>
@@ -13019,7 +13022,7 @@
         <v>5</v>
       </c>
       <c r="E127" s="3" t="s">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="F127" s="3" t="s">
         <v>273</v>
@@ -13030,10 +13033,10 @@
     </row>
     <row r="128" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A128" s="3" t="s">
-        <v>1128</v>
+        <v>1129</v>
       </c>
       <c r="B128" s="3" t="s">
-        <v>1129</v>
+        <v>1130</v>
       </c>
       <c r="C128" s="4">
         <v>3656</v>
@@ -13042,7 +13045,7 @@
         <v>5</v>
       </c>
       <c r="E128" s="3" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="F128" s="3" t="s">
         <v>273</v>
@@ -13096,10 +13099,10 @@
     </row>
     <row r="2" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1130</v>
+        <v>1131</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>1131</v>
+        <v>1132</v>
       </c>
       <c r="C2" s="4">
         <v>3459</v>
@@ -13108,7 +13111,7 @@
         <v>12</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
@@ -13119,10 +13122,10 @@
     </row>
     <row r="3" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1132</v>
+        <v>1133</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>1133</v>
+        <v>1134</v>
       </c>
       <c r="C3" s="4">
         <v>3803</v>
@@ -13131,7 +13134,7 @@
         <v>12</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>11</v>
@@ -13142,10 +13145,10 @@
     </row>
     <row r="4" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>1134</v>
+        <v>1135</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>1135</v>
+        <v>1136</v>
       </c>
       <c r="C4" s="4">
         <v>3425</v>
@@ -13154,10 +13157,10 @@
         <v>1</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="G4" s="4">
         <v>29</v>
@@ -13165,10 +13168,10 @@
     </row>
     <row r="5" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>1134</v>
+        <v>1135</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>1135</v>
+        <v>1136</v>
       </c>
       <c r="C5" s="4">
         <v>3426</v>
@@ -13177,7 +13180,7 @@
         <v>12</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>28</v>
@@ -13188,10 +13191,10 @@
     </row>
     <row r="6" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>1136</v>
+        <v>1137</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>1137</v>
+        <v>1138</v>
       </c>
       <c r="C6" s="4">
         <v>3427</v>
@@ -13200,10 +13203,10 @@
         <v>1</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="G6" s="4">
         <v>62.5</v>
@@ -13211,10 +13214,10 @@
     </row>
     <row r="7" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>1136</v>
+        <v>1137</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>1137</v>
+        <v>1138</v>
       </c>
       <c r="C7" s="4">
         <v>3428</v>
@@ -13223,7 +13226,7 @@
         <v>12</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>28</v>
@@ -13234,10 +13237,10 @@
     </row>
     <row r="8" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="C8" s="4">
         <v>3429</v>
@@ -13246,10 +13249,10 @@
         <v>1</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="G8" s="4">
         <v>76.5</v>
@@ -13257,10 +13260,10 @@
     </row>
     <row r="9" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="C9" s="4">
         <v>3430</v>
@@ -13269,7 +13272,7 @@
         <v>12</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>28</v>
@@ -13280,10 +13283,10 @@
     </row>
     <row r="10" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>1140</v>
+        <v>1141</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>1141</v>
+        <v>1142</v>
       </c>
       <c r="C10" s="4">
         <v>3913</v>
@@ -13292,10 +13295,10 @@
         <v>1</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="G10" s="4">
         <v>68</v>
@@ -13303,10 +13306,10 @@
     </row>
     <row r="11" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>1140</v>
+        <v>1141</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>1141</v>
+        <v>1142</v>
       </c>
       <c r="C11" s="4">
         <v>3872</v>
@@ -13315,7 +13318,7 @@
         <v>12</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>28</v>
@@ -13326,10 +13329,10 @@
     </row>
     <row r="12" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>1142</v>
+        <v>1143</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>1143</v>
+        <v>1144</v>
       </c>
       <c r="C12" s="4">
         <v>3422</v>
@@ -13338,10 +13341,10 @@
         <v>1</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="G12" s="4">
         <v>20</v>
@@ -13349,10 +13352,10 @@
     </row>
     <row r="13" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>1142</v>
+        <v>1143</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>1143</v>
+        <v>1144</v>
       </c>
       <c r="C13" s="4">
         <v>3423</v>
@@ -13361,7 +13364,7 @@
         <v>12</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>1144</v>
+        <v>1145</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>28</v>
@@ -13372,10 +13375,10 @@
     </row>
     <row r="14" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>1145</v>
+        <v>1146</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>1146</v>
+        <v>1147</v>
       </c>
       <c r="C14" s="4">
         <v>3431</v>
@@ -13384,10 +13387,10 @@
         <v>1</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="G14" s="4">
         <v>115</v>
@@ -13395,10 +13398,10 @@
     </row>
     <row r="15" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>1145</v>
+        <v>1146</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>1146</v>
+        <v>1147</v>
       </c>
       <c r="C15" s="4">
         <v>3432</v>
@@ -13407,7 +13410,7 @@
         <v>12</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>28</v>

</xml_diff>